<commit_message>
UI-parannus, domain-värit, varaneukkarit, multi-pass aikataulutus
- UnicaOne-fontti, taustakuva, hover-efektit, CSS-tooltipit
- Domain-värikoodaus tiimiselitteet.xlsx:stä, DOMAIN_ALIAS-mäppäys
- Varaneukkarit (Taka-Töölö, Etu-Töölö, Kaisaniemi, Laakso)
- Multi-pass aikataulutusalgoritmi: 5 strategiaa, paras valitaan
- Päivitetty Excel parsittu, nimimäppäykset korjattu
- Käännökset FI/EN, login-sivu, henkilöfiltteri auto-scroll

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
+++ b/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sanoma.sharepoint.com/sites/B2BGeneral667/Shared Documents/General/B2B (STEP) Cross-Domain Public/Seasonal Planning Process/2026_S3 materials/Dependency Synchronization Days/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9756CC9F-BADD-4AF6-BCC1-1EF6260770A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEE73A60-7162-4EA3-93BD-01488BFDAD5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{86D0FE88-11BB-614D-BBC1-5CCA99757B8D}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="18980" xr2:uid="{86D0FE88-11BB-614D-BBC1-5CCA99757B8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Synccipaltsu" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Synccipaltsu!$A$3:$J$55</definedName>
+    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">Synccipaltsu!$A$3:$J$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Synccipaltsu!$A$3:$J$58</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="180">
   <si>
     <t>S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08</t>
   </si>
@@ -96,12 +97,13 @@
     </r>
   </si>
   <si>
-    <t>Jaana Ty/Jaana Ta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Oma e2e arvotiimi tai ohjausryhmä (?) - input:ksi brief
-Filip Homberg, Jaanat, Jaakko Kuivalainen, Mikko Neva</t>
+    <t>Jaana Tynys</t>
+  </si>
+  <si>
+    <t>Filip Homberg, Jaana Tanskanen, Jaakko Kuivalainen, Mikko Neva</t>
+  </si>
+  <si>
+    <t>Oma e2e arvotiimi tai ohjausryhmä (?) - input:ksi brief</t>
   </si>
   <si>
     <t>S&amp;M</t>
@@ -140,9 +142,10 @@
 Heidi Falenius
 Satu Raatikainen
 Leena Koskinen
-DSE&amp;A: Vesa, Tanja, Jaana
-DG: Tuuli, Tuukka
-Print: Päivi
+DSE&amp;A: Vesa Lindqvist, Tanja Kaikkonen
+Jaana Tanskanen
+DG: Tuuli Rikama, Tuukka Antikainen
+Print: Päivi Vaittinen
 </t>
   </si>
   <si>
@@ -185,18 +188,17 @@
       <t xml:space="preserve">
 - kampanjaraportti
 - asiakastuki
-- palevlunhallinta Adnuntius</t>
-    </r>
-  </si>
-  <si>
-    <t>Toni Törnqvist 
-+ Sini Lähdemäki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DSE:  Bilal Gill, Heidi Falenius
-DG: Tuuli Rikama
-MSS: digitaalisten aineistobannereiden tuotanto - Weavy MCP?: Suvi Vesanen, Jani Moisiola
-</t>
+- palevlunhallinta Adnuntius, - consentin ja vendorlistin  päivitys</t>
+    </r>
+  </si>
+  <si>
+    <t>Tuuli Rikama</t>
+  </si>
+  <si>
+    <t>DSE: Bilal Gill, Heidi Falenius, Juho Pöyhönen, Maiju Häkkinen
+DG: Anniina Hautala, Toni Törnqvist, Janne Mikkola, Sini Lähdemäki, Birgitta Kursi, Anu Ollikainen, Rosa Forsell, Jonne Ansamaa, Airi Viljamaa, Mikko Vartiainen
+MSS: Suvi Vesanen, Jani Moisiola
+TM: Päivi Vaittinen, Niina Grönholm</t>
   </si>
   <si>
     <r>
@@ -223,7 +225,13 @@
     </r>
   </si>
   <si>
-    <t>Ensin kaupallinen keskustelu, jonka jälkeen tekninen arvio. Arkkitehtuuri huomioiden (Filip ja Co)</t>
+    <t>Jaana Tanskanen</t>
+  </si>
+  <si>
+    <t>Filip Holmberg, Jaana Tynys</t>
+  </si>
+  <si>
+    <t>Ensin kaupallinen keskustelu, jonka jälkeen tekninen arvio. Arkkitehtuuri huomioiden.</t>
   </si>
   <si>
     <r>
@@ -256,12 +264,13 @@
     <t>Heidi Falenius</t>
   </si>
   <si>
-    <t xml:space="preserve">DSE: Antero Karttunen, Vesa Lindqvist
-DG: Anniina Hautala, Toni Törnqvist, Airi Viljamaa, Janne Mikkonen,…
-MSS (monimediallinen aineistotuotanto - print aineistobannereiden tuotanto digi bannerista(?)): Suvi Vesanen, Jani Moisiola
+    <t>DSE: Antero Karttunen, Vesa Lindqvist
+DG: Anniina Hautala, Toni Törnqvist, Airi Viljamaa, Janne Mikkonen, Sini Lähdemäki
+MSS: Suvi Vesanen, Jani Moisiola
 TM: Päivi Vaittiinen, Harri Lilja
 N&amp;F: Sanna Wirkkala
-</t>
+Jaana Tanskanen
+Jero Liimatainen</t>
   </si>
   <si>
     <t>MSS</t>
@@ -307,9 +316,9 @@
     <t>Jani Moisiola
 Sami Vallius
 Mikko Laine
-Bilal Gill?
-Aleksandrs Breus?
-Monday: Johannes Ojala / Cristian Ramirez?</t>
+Bilal Gill
+Aleksandrs Breus
+Johannes Ojala / Cristian Ramirez</t>
   </si>
   <si>
     <t>1h</t>
@@ -326,7 +335,7 @@
 Anniina Hautala
 Filip Holmberg
 Jaana Tanskanen
-SF/Advendio tuotehallinta/laskutus Heidi Falenius</t>
+Heidi Falenius</t>
   </si>
   <si>
     <t>Insight&amp;Research -tiimin Monday-käyttöönotto</t>
@@ -355,9 +364,6 @@
 Sami Vallius</t>
   </si>
   <si>
-    <t>MSS / SM</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -382,7 +388,7 @@
     </r>
   </si>
   <si>
-    <t>MS&amp;S: Sari Kärki, Jaana Jamalainen
+    <t>MS&amp;S: Sari Kärki, Jaana Jamalainen, Tarja Viljanen
 S&amp;M: Hanna Jalonen, Tiina Virtanen</t>
   </si>
   <si>
@@ -391,6 +397,9 @@
   </si>
   <si>
     <t>- Avauksen rooli: Terhi+Ossi?</t>
+  </si>
+  <si>
+    <t>ei suunnittelua</t>
   </si>
   <si>
     <t>DSE Prio 10: Yhteinen kaupallinen johtamismalli/RevOps: Yhteisen kaupallisen johtamismallin luonti ja käyttöönotto pienemmän asiakassegmentin osalta (RevOps) ja markkinoinnin yhteistyön selkeyttäminen osana kompetenssityötä</t>
@@ -457,20 +466,20 @@
     <t>Sami Luutikivi</t>
   </si>
   <si>
-    <t xml:space="preserve">Digital &amp; AI: Sami Luutikivi, Mikko Neva?, Filip Holmberg
+    <t xml:space="preserve">Digital &amp; AI: Sami Luutikivi, Mikko Neva, Filip Holmberg
 Core &amp; Sales Reporting: </t>
   </si>
   <si>
-    <t>S&amp;M/B2B</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tuloksellisuus. Asiakaslähtöisen tuotehierarkian kerroksen luominen asiakasrajapintaan konseptin mukaisesti (huomioiden päivittynyt/päivittyvä strategia ja mainoskokemuksen korostunut rooli). Ns. "konepelti" - ei kosketa tuotehierarkiaan tällä sesongilla konepellin alla). </t>
   </si>
   <si>
-    <t>Hanna Jalonen</t>
-  </si>
-  <si>
-    <t>Tuotemyynti, markkinointi, admanager -  osallistujat tarkennetaan tiistaina. Tuomo Sinkkonen, Lotta Monten, Minna Kruhse, Riku Talvitie, Janne Nurmisto, Vesa Lindqvist, Maiju Häkkinen, Leena Koskinen</t>
+    <t>Leena Koskinen &amp; Tuomo Sinkkonen</t>
+  </si>
+  <si>
+    <t>Janne Nurmisto,  Tuomo Sinkkonen, Lotta Monten, Minna Kruhse, Riku Talvitie, Leena Koskinen, Tiina Kosonen, Hanna Jalonen</t>
+  </si>
+  <si>
+    <t>Tämä ti 13-14 Product Sales tiimiksen aikaan (buukattu)</t>
   </si>
   <si>
     <t>Tuloksellisuus. Tavoite ja mittarimallin seuraavat vaiheet &amp; vaikutukset eri domaineille (odotukset painottuen S1, mutta domainien odotetaan arvioivan ja huomioivan vaikutuksia jo S3 nykyisessä tekemisessä)</t>
@@ -479,34 +488,43 @@
     <t>Tiina Kosonen</t>
   </si>
   <si>
-    <t>Vaiheen 1 toimenpiteisiin liittyvät henkilöt eri domaineista. Tarkennetaan tiistaina</t>
+    <t>Maria Meurman (DSE), Mikko Neva (DSE), Filip Holmberg (Architecture), Kati Alijoki (osaamisen kehittäminen), Leena Koskinen (markkinointi), Jonne Ansamaa (raportointi), Jenni Tamminen (Kasvupalvelu), Vesa Lindqvist (Admanager), Jaana Tanskanen (optio)</t>
   </si>
   <si>
     <t>Tuloksellisuus. Yhteiskehittämisen mallin edistäminen S3. Valitut end-to-end yhteiskehittämisen mallin mukaiset pilotit (revops &amp; tuloksellisuuden malli). Miten data tallennetaan, varmistetaan, että toimitaan S3 mallin edistämiseksi fiksusti vaikka sen ympärillä ei teknisempää kehitystä.</t>
   </si>
   <si>
-    <t>tiistaina tarkentuu. Tiina Virtanen (Solutions Sales), Sami Tirkkonen (CX), Hanna Jalonen (Salesdev), Sami Luutiviki (data)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strateginen segmentointi ja ICP - vaiheen 2 toteutus. </t>
-  </si>
-  <si>
-    <t>Juhana Rautavirta, Tiina Kosonen, Hanna Jalonen, Eetu Laitinen, Perttu Rekola, Maiju Häkkinen, markkinointi  Leena palaa kuka markkinoinnista</t>
+    <t>Reeta Thurman (Markkinointistrategt), Tiina Virtanen (Solutions Sales), Pilvi Seppälä (Sales dev), Sami Tirkkonen (CX), Hanna Jalonen (Salesdev), Sami Luutiviki (data)</t>
+  </si>
+  <si>
+    <t>0,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Strateginen segmentointi) ICP:n eli ideal customer profilen luominen </t>
+  </si>
+  <si>
+    <t>Leena Koskinen, Juhana Rautavirta, Tiina Kosonen, Hanna Jalonen, Eetu Laitinen, Perttu Rekola, Maiju Häkkinen</t>
+  </si>
+  <si>
+    <t>ti 10.30-13 välillä tai ke</t>
   </si>
   <si>
     <t>Discovery: jatkuvat palvelutuotteet varattaviksi (Kasvupalvelu Startti, Google, Meta)</t>
   </si>
   <si>
-    <t>Jenni Tammninen</t>
-  </si>
-  <si>
-    <t>Heidi Falenius, TBD</t>
+    <t>Jenni Tamminen</t>
+  </si>
+  <si>
+    <t>Heidi Falenius, Maria Meurman (offertool), Marja Laulainen</t>
   </si>
   <si>
     <t>Discovery: kasvupalvelun suunnittelutiimin työkalujen ja järjestelmien pienkehitystyö ja suunnittelu miten kannattaisi hyödyntää esim. SalesForcea</t>
   </si>
   <si>
-    <t>Filip Holmberg, Jaana Tanskanen, Jonne Ansamaa</t>
+    <t>Filip Holmberg, Jaana Tanskanen, Jonne Ansamaa, Nea Särkikoski, Niko-Petteri Varho</t>
+  </si>
+  <si>
+    <t>Ei dep syncciin. Toive, että 1vk myöhemmin</t>
   </si>
   <si>
     <t>Discovery: kasvupalvelun asiakkaiden mainosdatan rikastaminen tulosten parantamiseksi; vaihtoehtojen kartoitus ja pilotointi. Datan parannus melko domainin sisäinen työ, mutta pitää huomioida raportointi ja datayhteys näkökulmasta</t>
@@ -515,16 +533,22 @@
     <t>John Kronström, TBD</t>
   </si>
   <si>
+    <t>Ei dep syncciin. Toive, että 2vk myöhemmin</t>
+  </si>
+  <si>
     <t>Kasvuraportin kehitystyö, jatkokehitys (pienkehitys)</t>
   </si>
   <si>
     <t>TBD</t>
   </si>
   <si>
+    <t>Ei dep syncciin.</t>
+  </si>
+  <si>
     <t>Discovery: verkkokauppasegmentin tuotemahdollisuudet</t>
   </si>
   <si>
-    <t>TBD
+    <t>Ida Soini
 DG: Tuuli Rikama, Tuukka Antikainen</t>
   </si>
   <si>
@@ -551,27 +575,23 @@
 MSS Insight: Jaana Jamalainen</t>
   </si>
   <si>
-    <t>AI Platform &amp; Operating model
-- API uudistuksen PoC tukemaan AI kehitystä</t>
+    <t>API uudistuksen PoC tukemaan AI kehitystä</t>
   </si>
   <si>
     <t>Filip Holmberg</t>
   </si>
   <si>
-    <t>Filip
-Digital &amp; AI: Jero, Heidi Falenius
-Core &amp; Sales Reporting: Bilal
-(DSE&amp;A: Rolf Sormo --&gt; ajatuksia tekniseen malliin suunnittelussa)</t>
-  </si>
-  <si>
-    <t>Yhteinen kaupallinen johtamismalli: 
-- prospektoinnin ja skoutti pelikaverin kehittäminen</t>
-  </si>
-  <si>
-    <t>Sales Dev: Antti Ovaska, Juhana Rautavirta, Tiina Kosonen DSE: Maria Meurman, Vesa Lindqvist</t>
+    <t>Digital &amp; AI: Jero Liimatainen, Heidi Falenius
+Core &amp; Sales Reporting: Antero Karttunen,  Bilal Gill</t>
+  </si>
+  <si>
+    <t>B2B</t>
   </si>
   <si>
     <t>TagomoAI agenttinen Ad Manager bookkaus: Toiminnallisuus, jossa automaagisesti päivitettään agency-advertiser relaatiota tiettyjen toimistojen osalta.</t>
+  </si>
+  <si>
+    <t>Hanna Jalonen</t>
   </si>
   <si>
     <t>Jaana Tanskanen/Filip Holmberg
@@ -586,7 +606,7 @@
     <t>Janne Nikkilä</t>
   </si>
   <si>
-    <t>Digital &amp; AI: Abhaya
+    <t>Digital &amp; AI: Abhaya Pani
 Core &amp; Sales Reporting: Marko Ukkola
 DG: Janne Eränen</t>
   </si>
@@ -616,7 +636,7 @@
     <t>Toni Törnqvist</t>
   </si>
   <si>
-    <t xml:space="preserve">Ad Manager (Toni/Tuomas, Janne, Anniina) &amp; Creative AI (Sini, Asko, Airi)
+    <t xml:space="preserve">Ad Manager (Toni Törnqvist, Tuomas Waris, Janne Mikkonen, Anniina Hautala) &amp; Creative AI (Sini Lähdemäki, Asko Sälli, Airi Viljamaa)
 </t>
   </si>
   <si>
@@ -669,7 +689,18 @@
     <t>Emmy Ramsay</t>
   </si>
   <si>
-    <t>Ad Manager Product, Campaign Performance &amp; Reporting, DSE Core, Digital Operations, Product Sales, Marketing, Performance Products, Sales Development Team</t>
+    <t>Ad Manager Product: Anniina Hautala, Toni Törnqvist
+Campaign Performance &amp; Reporting: Jonne Ansamaa, Pilvi Rimmanen
+DSE Core: Heidi Falenius
+Airi Viljamaa, Juho Pöyhönen
+Creative AI: Sini Lähdemäki​
+DSEA: Vesa Lindqvist
+Digital Operations: Anu Ollikainen
+Product Sales: Minna Kruhse
+Marketing: Ritva Lassila
+Performance Products: Johannes Hocksell
+Sales Development Team: Hanna Jalonen, Tiina Kosonen
+YDP: Maiju Toivonen, Netta Aavikko, Tuukka Antikainen, Johan Korsbäck</t>
   </si>
   <si>
     <r>
@@ -680,7 +711,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Insteram to Ad Manager </t>
+      <t xml:space="preserve">Instream to Ad Manager </t>
     </r>
     <r>
       <rPr>
@@ -693,10 +724,10 @@
     </r>
   </si>
   <si>
-    <t>TM: Anu, Teemu, Laura
-DG: Toni/Tuomas, Anniina, Janne
-MSS: Raatikainen Satu (toimisto kulma) ?
-DSE: joku CS tiimistä asiakkaan näkökulmaa tuomaan?
+    <t>TM: Anu Linden, Teemu Ihalainen, Laura KAngas
+DG: Toni Törnqvist, Tuomas Waris, Anniina Hautala, Janne Mikkonen
+MSS: Raatikainen Satu (toimisto kulma)
+DSE: joku CS tiimistä asiakkaan näkökulmaa tuomaan (Maiju tai hänen nimeämä henkilö)?
 Sami Malmi</t>
   </si>
   <si>
@@ -814,6 +845,9 @@
     </r>
   </si>
   <si>
+    <t>Ei dep syncciin</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -839,11 +873,11 @@
     <t>Netta Aavikko</t>
   </si>
   <si>
-    <t>Ad Manager Product, Campaign Performance &amp; Reporting, Performance Products, Product Sales, Marketing, DSE Core, Digital Operations
+    <t>Ad Manager Product, Campaign Performance &amp; Reporting, Performance Products, Product Sales, Marketing, DSE Core Heidi Falenius, Digital Operations
 PP: Johannes Hocksell
 CPR: Janne Eränen, Jonne Ansamaa​
 Juho Pöyhönen
-YDP: Mikko Vartiainen, Emmy Ramsay, Maiju Toivinen
+YDP: Mikko Vartiainen, Emmy Ramsay, Maiju Toivonen
 Ad Manager Product: Toni Törnqvist, Anniina Hautala
 Marketing: Ritva Lassila</t>
   </si>
@@ -871,16 +905,37 @@
     <t>Zahoor Khan</t>
   </si>
   <si>
-    <t>Creative AI, Ad Manager Product, CPR</t>
-  </si>
-  <si>
-    <t>Data Product work</t>
+    <t xml:space="preserve">Creative AI: Asko Sälli,Zeeshan Rais, CPR: Janne Eränen (for collecting campaign data for those video creatives from snowflake). OPU: Martti Halme (For snowplow pixel data that lands in Snowflake), Netta Aavikko  </t>
+  </si>
+  <si>
+    <t>1.5h</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data Product work - </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>huom! Varmistetaan Data Council ohjausmalli "miten" tehdään on huomioituna suunnittelussa</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
   <si>
     <t>Jonne Ansamaa</t>
-  </si>
-  <si>
-    <t>DG/B2B</t>
   </si>
   <si>
     <t xml:space="preserve">Optimizing the flow between Snowflake and Claude </t>
@@ -917,19 +972,103 @@
 BSS Sales​</t>
   </si>
   <si>
-    <t>AV  Maestro</t>
+    <t>AV  Maestro, meeting 1</t>
   </si>
   <si>
     <t>Panu Hyryläinen</t>
   </si>
   <si>
-    <t>Campaign performance &amp; Reporting, Total TV &amp; Audio Operations &amp; Self Service, Nelonen Media, Nelonen Media (Radio), B2B API Team?B2B Core &amp; Sales Reporting Mission Team​?, Creative AI (Sini), External partner (IX), External partner (MediaTailor - MediaPocket expert)</t>
-  </si>
-  <si>
-    <t>3 h</t>
-  </si>
-  <si>
-    <t>dep.sync</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>AV Maestro - B2B Core &amp; Sales Reporting Mission Team​</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve"> (60 min)
+Panu Hyryläinen, Annika Palm, Joonas Imeläinen, Anu Linden, Pia Viinikainen, Heidi Falenius, Juho Pöyhönen, Antero Karttunen</t>
+    </r>
+  </si>
+  <si>
+    <t>tulee dep.sync</t>
+  </si>
+  <si>
+    <t>AV  Maestro, meeting 2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">AV Maestro - Campaign Performance &amp; Reporting </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>(60 min)
+Panu Hyryläinen, Annika Palm, Joonas Imeläinen, Mikko Eskelinen, Tina Åström, Anu Linden, Sari Moilanen, Jonne Ansamaa, Janne Eränen</t>
+    </r>
+  </si>
+  <si>
+    <t>AV  Maestro, meeting 3</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>AV Maestro - Total TV and Audio Operations &amp; Self Service</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve"> (60 min)
+Panu Hyryläinen, Annika Palm, Joonas Imeläinen, Mari Härkisaari, Erik Keski-Ojala
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve">AV Maestro – Creative AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>(30 min)
+Panu Hyryläinen, Annika Palm, Joonas Imeläinen, Sini Lähdemäki, Airi Viljamaa</t>
+    </r>
+  </si>
+  <si>
+    <t>30min</t>
   </si>
   <si>
     <t>AV Manager, rahapelaaminen, tuotteiden konfigurointi &amp; myynnin rajoitteet</t>
@@ -938,7 +1077,7 @@
     <t>Anu Linden</t>
   </si>
   <si>
-    <t>Sales Engine Transformation: Hedi Falenius,  Juho Pöyhönen, Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Teemu Ihalainen, Sina Reunala, Petri Lahikainen, Roope Hämäläinen</t>
+    <t>B2B Core: Hedi Falenius,  Juho Pöyhönen, Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Teemu Ihalainen, Sina Reunala, Petri Lahikainen, Roope Hämäläinen</t>
   </si>
   <si>
     <t>2 h</t>
@@ -958,21 +1097,21 @@
 DSE Heidi Falenius</t>
   </si>
   <si>
-    <t>Muuten konfigurointia ja sopimista, mutta käsitellään rahapelaamisen osuus omassaan AV Managerin alla.</t>
-  </si>
-  <si>
-    <t>TV Beat</t>
-  </si>
-  <si>
-    <t>Total TV &amp; Audio Operations &amp; Self Service​
-DG: Campaign performance &amp; Reporting​: Jonne Ansamaa, Sari Moilanen 
-DSE Sales Engine Architecture &amp; Transformation Filip Holmberg, Bilal Gill</t>
-  </si>
-  <si>
-    <t>1 h</t>
-  </si>
-  <si>
-    <t>B2B</t>
+    <t>ei tarvita palaveria, ei dep syncciin</t>
+  </si>
+  <si>
+    <t>TV Beat, meeting 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV Beat (1 h)
+Sari Moilanen, Jonne Ansamaa, Janne Eränen, Mikko Eskelinen, Panu Hyryläinen, Tapani Kuokkanen, Erik Keski-Ojala, Pasi Korhonen. </t>
+  </si>
+  <si>
+    <t>TV Beat, meeting 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV Beat Core (30 min)
+Heidi Falenius, Juho Pöyhönen, Bilal Gill, Mikko Eskelinen, Panu Hyryläinen. </t>
   </si>
   <si>
     <t>SMF tieto-omaisuuden (”data”) hallinta ja kehitys B2B:n näkökulmasta. Aloitetaan natiivin tukemisesta.​</t>
@@ -987,13 +1126,19 @@
     <t>Campaign performance &amp; Reporting: Jonne Ansamaa, Riia Luhtala, Sari Moilanen, Pilvi Rimmanen
 Core &amp; Sales Reporting: Heidi Falenius, Sampsa Näkki. 
 Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Pia Viinikainen, Joonas Imeläinen, Teemu Ihalainen, Petri Lahikainen, Mikko Eskelinen, Panu Hyryläinen, Sina Reunala, Laura Kangas, Tina Åström</t>
+  </si>
+  <si>
+    <t>3 h</t>
+  </si>
+  <si>
+    <t>dep.sync</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25">
+  <fonts count="29">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1042,13 +1187,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
@@ -1079,12 +1217,6 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1119,7 +1251,13 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1134,12 +1272,12 @@
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1152,6 +1290,40 @@
     <font>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
@@ -1249,7 +1421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1289,13 +1461,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1312,14 +1479,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1329,28 +1488,31 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1364,23 +1526,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -1389,17 +1545,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1409,52 +1556,88 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1832,19 +2015,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07127F19-9F63-3B48-ABE6-8FC4ADCB9798}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:J66"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:J69"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="3.125" style="39" customWidth="1"/>
+    <col min="1" max="1" width="3" style="37" customWidth="1"/>
     <col min="2" max="2" width="9" style="2" customWidth="1"/>
     <col min="3" max="3" width="11" style="2"/>
-    <col min="4" max="4" width="70.5" customWidth="1"/>
+    <col min="4" max="4" width="87.5" customWidth="1"/>
     <col min="5" max="5" width="18.875" style="34" customWidth="1"/>
     <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="16.5" customWidth="1"/>
-    <col min="8" max="8" width="15.125" customWidth="1"/>
-    <col min="9" max="9" width="22.625" customWidth="1"/>
+    <col min="7" max="7" width="18.625" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="31.5" customWidth="1"/>
     <col min="10" max="10" width="15.5" style="34" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1853,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30.75">
+    <row r="3" spans="1:10" ht="32.1">
       <c r="B3" s="32" t="s">
         <v>1</v>
       </c>
@@ -1882,1426 +2064,1531 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A4" s="40"/>
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="38.25">
+      <c r="A4" s="38"/>
       <c r="B4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="44">
+      <c r="C4" s="15">
         <v>11</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="22" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="20"/>
-      <c r="H4" s="15" t="b">
+      <c r="H4" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I4" s="16"/>
+      <c r="I4" s="16" t="s">
+        <v>14</v>
+      </c>
       <c r="J4" s="34"/>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="126">
-      <c r="A5" s="40"/>
-      <c r="B5" s="45" t="s">
-        <v>14</v>
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="165">
+      <c r="A5" s="38"/>
+      <c r="B5" s="42" t="s">
+        <v>15</v>
       </c>
       <c r="C5" s="14">
         <v>2</v>
       </c>
-      <c r="D5" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="24" t="s">
+      <c r="D5" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="E5" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15" t="b">
+      <c r="F5" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="22"/>
+      <c r="H5" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="64"/>
       <c r="J5" s="34"/>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="117">
-      <c r="A6" s="40"/>
-      <c r="B6" s="45" t="s">
-        <v>18</v>
+    <row r="6" spans="1:10" s="1" customFormat="1" ht="128.1" customHeight="1">
+      <c r="A6" s="38"/>
+      <c r="B6" s="42" t="s">
+        <v>19</v>
       </c>
       <c r="C6" s="14">
         <v>2</v>
       </c>
-      <c r="D6" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="E6" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="14"/>
-      <c r="H6" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="I6" s="38"/>
+      <c r="F6" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="22">
+        <v>3</v>
+      </c>
+      <c r="H6" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="64"/>
       <c r="J6" s="34"/>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A7" s="40"/>
-      <c r="B7" s="45" t="s">
+    <row r="7" spans="1:10" s="1" customFormat="1" ht="77.25">
+      <c r="A7" s="38"/>
+      <c r="B7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="14">
         <v>2</v>
       </c>
-      <c r="D7" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="37" t="s">
+      <c r="D7" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15" t="b">
+      <c r="E7" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="22"/>
+      <c r="H7" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="38"/>
+      <c r="I7" s="64" t="s">
+        <v>26</v>
+      </c>
       <c r="J7" s="34"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="90.95">
-      <c r="A8" s="40"/>
-      <c r="B8" s="45" t="s">
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="105">
+      <c r="A8" s="38"/>
+      <c r="B8" s="42" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="14">
         <v>2</v>
       </c>
-      <c r="D8" s="25" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="14"/>
-      <c r="H8" s="15" t="b">
+      <c r="D8" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="22"/>
+      <c r="H8" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="38"/>
-      <c r="J8" s="34"/>
-    </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="78">
-      <c r="A9" s="40"/>
-      <c r="B9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="41" t="s">
+      <c r="I8" s="64"/>
+      <c r="J8" s="70"/>
+    </row>
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="99" customHeight="1">
+      <c r="A9" s="38"/>
+      <c r="B9" s="26" t="s">
         <v>30</v>
       </c>
+      <c r="C9" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="39" t="s">
+        <v>33</v>
+      </c>
       <c r="F9" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" s="15" t="b">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="71" t="b">
+        <v>1</v>
       </c>
       <c r="I9" s="16"/>
       <c r="J9" s="34"/>
     </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="78">
-      <c r="A10" s="40"/>
+    <row r="10" spans="1:10" s="1" customFormat="1" ht="96.95" customHeight="1">
+      <c r="A10" s="38"/>
       <c r="B10" s="30" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C10" s="14">
         <v>9</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10"/>
+      <c r="H10" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="16"/>
+      <c r="J10" s="34"/>
+    </row>
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="38.25">
+      <c r="A11" s="38"/>
+      <c r="B11" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="15">
+        <v>10</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="G10"/>
-      <c r="H10" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="I10" s="13"/>
-      <c r="J10" s="34"/>
-    </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A11" s="40"/>
-      <c r="B11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="44">
-        <v>10</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="14"/>
-      <c r="H11" s="15" t="b">
-        <v>0</v>
+      <c r="H11" s="33" t="b">
+        <v>1</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="34" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A12" s="40"/>
+      <c r="A12" s="38"/>
       <c r="B12" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="24"/>
-      <c r="D12" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>41</v>
+        <v>30</v>
+      </c>
+      <c r="C12" s="23"/>
+      <c r="D12" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>44</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="14"/>
-      <c r="H12" s="15" t="b">
+        <v>45</v>
+      </c>
+      <c r="G12" s="22"/>
+      <c r="H12" s="33" t="b">
         <v>0</v>
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A13" s="40"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A13" s="38"/>
       <c r="B13" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="24">
+        <v>30</v>
+      </c>
+      <c r="C13" s="23">
         <v>7</v>
       </c>
-      <c r="D13" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>37</v>
+      <c r="D13" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>40</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="23"/>
+        <v>47</v>
+      </c>
+      <c r="G13" s="22"/>
       <c r="H13" s="33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="34"/>
     </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A14" s="40"/>
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="30">
+      <c r="A14" s="38"/>
       <c r="B14" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="23">
         <v>11</v>
       </c>
-      <c r="D14" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="24"/>
-      <c r="F14" s="42" t="s">
-        <v>47</v>
-      </c>
-      <c r="G14" s="23"/>
+      <c r="D14" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="23"/>
+      <c r="F14" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="22"/>
       <c r="H14" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I14" s="16"/>
+      <c r="I14" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="J14" s="34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A15" s="40"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="30">
+      <c r="A15" s="38"/>
       <c r="B15" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="23">
         <v>10</v>
       </c>
-      <c r="D15" s="46" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="43" t="s">
-        <v>49</v>
-      </c>
-      <c r="G15" s="14"/>
-      <c r="H15" s="15" t="b">
+      <c r="D15" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="E15" s="22"/>
+      <c r="F15" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="22"/>
+      <c r="H15" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I15" s="28"/>
+      <c r="I15" s="27"/>
       <c r="J15" s="34" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A16" s="40"/>
+      <c r="A16" s="38"/>
       <c r="B16" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="23">
         <v>10</v>
       </c>
-      <c r="D16" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="F16" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="G16" s="14"/>
-      <c r="H16" s="15" t="b">
+      <c r="D16" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" s="22"/>
+      <c r="H16" s="33" t="b">
         <v>1</v>
       </c>
-      <c r="I16" s="28"/>
+      <c r="I16" s="27"/>
       <c r="J16" s="34"/>
     </row>
     <row r="17" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A17" s="40"/>
-      <c r="B17" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="44">
+      <c r="A17" s="38"/>
+      <c r="B17" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="15">
         <v>4</v>
       </c>
-      <c r="D17" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>54</v>
+      <c r="D17" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>57</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="G17" s="14"/>
-      <c r="H17" s="21" t="b">
+        <v>58</v>
+      </c>
+      <c r="G17" s="22"/>
+      <c r="H17" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I17" s="17"/>
       <c r="J17" s="29"/>
     </row>
     <row r="18" spans="1:10" s="1" customFormat="1" ht="51.95">
-      <c r="A18" s="40"/>
-      <c r="B18" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="47" t="s">
-        <v>56</v>
+      <c r="A18" s="38"/>
+      <c r="B18" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>59</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>61</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" s="14"/>
-      <c r="H18" s="15" t="b">
+        <v>62</v>
+      </c>
+      <c r="G18" s="22"/>
+      <c r="H18" s="33" t="b">
         <v>0</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="34"/>
     </row>
     <row r="19" spans="1:10" s="1" customFormat="1" ht="51.95">
-      <c r="A19" s="40"/>
-      <c r="B19" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="47" t="s">
-        <v>56</v>
+      <c r="A19" s="38"/>
+      <c r="B19" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="62" t="s">
+        <v>59</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>58</v>
+        <v>63</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>61</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" s="14"/>
-      <c r="H19" s="15" t="b">
+        <v>64</v>
+      </c>
+      <c r="G19" s="22"/>
+      <c r="H19" s="33" t="b">
         <v>1</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J19" s="34"/>
     </row>
-    <row r="20" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A20" s="40"/>
+    <row r="20" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A20" s="38"/>
       <c r="B20" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>64</v>
+      <c r="C20" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>67</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="G20" s="14"/>
-      <c r="H20" s="15" t="b">
+        <v>68</v>
+      </c>
+      <c r="G20" s="22"/>
+      <c r="H20" s="33" t="b">
         <v>0</v>
       </c>
       <c r="I20" s="16"/>
       <c r="J20" s="34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A21" s="40"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" s="1" customFormat="1" ht="51.95">
+      <c r="A21" s="38"/>
       <c r="B21" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C21" s="24">
+        <v>15</v>
+      </c>
+      <c r="C21" s="23">
         <v>1</v>
       </c>
-      <c r="D21" s="36" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>68</v>
+      <c r="D21" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>70</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" s="14">
+        <v>71</v>
+      </c>
+      <c r="G21" s="22">
         <v>1</v>
       </c>
-      <c r="H21" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I21" s="16"/>
-      <c r="J21" s="34"/>
+      <c r="H21" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" s="34" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="22" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A22" s="40"/>
+      <c r="A22" s="38"/>
       <c r="B22" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="24">
+        <v>15</v>
+      </c>
+      <c r="C22" s="23">
         <v>1</v>
       </c>
-      <c r="D22" s="36" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>71</v>
+      <c r="D22" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>74</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="G22" s="14">
+        <v>75</v>
+      </c>
+      <c r="G22" s="22">
         <v>1</v>
       </c>
-      <c r="H22" s="21" t="b">
+      <c r="H22" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I22" s="16"/>
       <c r="J22" s="34"/>
     </row>
     <row r="23" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A23" s="40"/>
+      <c r="A23" s="38"/>
       <c r="B23" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" s="24">
+        <v>15</v>
+      </c>
+      <c r="C23" s="23">
         <v>1</v>
       </c>
-      <c r="D23" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>71</v>
+      <c r="D23" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" s="22" t="s">
+        <v>74</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="G23" s="14">
-        <v>0.5</v>
-      </c>
-      <c r="H23" s="21" t="b">
-        <v>0</v>
+        <v>77</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="43" t="b">
+        <v>1</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="34"/>
     </row>
     <row r="24" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A24" s="40"/>
+      <c r="A24" s="38"/>
       <c r="B24" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="24">
+        <v>15</v>
+      </c>
+      <c r="C24" s="23">
         <v>1</v>
       </c>
-      <c r="D24" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="23"/>
+      <c r="D24" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>74</v>
+      </c>
       <c r="F24" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="G24" s="14">
+        <v>80</v>
+      </c>
+      <c r="G24" s="22">
         <v>1</v>
       </c>
-      <c r="H24" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I24" s="16"/>
+      <c r="H24" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" s="16" t="s">
+        <v>81</v>
+      </c>
       <c r="J24" s="34"/>
     </row>
-    <row r="25" spans="1:10" s="1" customFormat="1" ht="15.95">
-      <c r="A25" s="40"/>
+    <row r="25" spans="1:10" s="1" customFormat="1">
+      <c r="A25" s="38"/>
       <c r="B25" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="24">
+        <v>15</v>
+      </c>
+      <c r="C25" s="23">
         <v>9</v>
       </c>
-      <c r="D25" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>78</v>
+      <c r="D25" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>83</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="21" t="b">
+        <v>84</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="34"/>
     </row>
-    <row r="26" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A26" s="40"/>
+    <row r="26" spans="1:10" s="1" customFormat="1" ht="25.5">
+      <c r="A26" s="38"/>
       <c r="B26" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C26" s="24">
+        <v>15</v>
+      </c>
+      <c r="C26" s="23">
         <v>9</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>78</v>
+        <v>85</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>83</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="G26" s="14"/>
-      <c r="H26" s="21" t="b">
+        <v>86</v>
+      </c>
+      <c r="G26" s="22"/>
+      <c r="H26" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I26" s="16"/>
+      <c r="I26" s="16" t="s">
+        <v>87</v>
+      </c>
       <c r="J26" s="34"/>
     </row>
-    <row r="27" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A27" s="40"/>
+    <row r="27" spans="1:10" s="1" customFormat="1" ht="25.5">
+      <c r="A27" s="38"/>
       <c r="B27" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C27" s="24">
+        <v>15</v>
+      </c>
+      <c r="C27" s="23">
         <v>9</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>78</v>
+        <v>88</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>83</v>
       </c>
       <c r="F27" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G27" s="22"/>
+      <c r="H27" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="J27" s="34"/>
+    </row>
+    <row r="28" spans="1:10" s="1" customFormat="1" ht="15.75">
+      <c r="A28" s="38"/>
+      <c r="B28" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="23">
+        <v>9</v>
+      </c>
+      <c r="D28" s="63" t="s">
+        <v>91</v>
+      </c>
+      <c r="E28" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G27" s="14"/>
-      <c r="H27" s="21" t="b">
+      <c r="F28" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="G28" s="22"/>
+      <c r="H28" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I27" s="16"/>
-      <c r="J27" s="34"/>
-    </row>
-    <row r="28" spans="1:10" s="1" customFormat="1" ht="15.95">
-      <c r="A28" s="40"/>
-      <c r="B28" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C28" s="24">
+      <c r="I28" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="J28" s="34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" s="1" customFormat="1" ht="26.1">
+      <c r="A29" s="38"/>
+      <c r="B29" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="23">
         <v>9</v>
       </c>
-      <c r="D28" s="64" t="s">
-        <v>84</v>
-      </c>
-      <c r="E28" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="G28" s="14"/>
-      <c r="H28" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I28" s="16"/>
-      <c r="J28" s="34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" s="1" customFormat="1" ht="26.1">
-      <c r="A29" s="40"/>
-      <c r="B29" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="24">
-        <v>9</v>
-      </c>
-      <c r="D29" s="64" t="s">
-        <v>86</v>
-      </c>
-      <c r="E29" s="23" t="s">
-        <v>78</v>
+      <c r="D29" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="E29" s="22" t="s">
+        <v>83</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="G29" s="14"/>
-      <c r="H29" s="21" t="b">
+        <v>95</v>
+      </c>
+      <c r="G29" s="22"/>
+      <c r="H29" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="34"/>
     </row>
-    <row r="30" spans="1:10" s="1" customFormat="1" ht="78.75" customHeight="1">
-      <c r="A30" s="40"/>
-      <c r="B30" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C30" s="44">
+    <row r="30" spans="1:10" s="1" customFormat="1" ht="51.95">
+      <c r="A30" s="38"/>
+      <c r="B30" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="15">
         <v>5</v>
       </c>
-      <c r="D30" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="E30" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="F30" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="G30" s="14"/>
-      <c r="H30" s="21" t="b">
+      <c r="D30" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="F30" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="G30" s="22"/>
+      <c r="H30" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I30" s="26"/>
+      <c r="I30" s="36"/>
       <c r="J30" s="29"/>
     </row>
-    <row r="31" spans="1:10" s="1" customFormat="1" ht="66.75" customHeight="1">
-      <c r="A31" s="40"/>
-      <c r="B31" s="27" t="s">
+    <row r="31" spans="1:10" s="1" customFormat="1" ht="39">
+      <c r="A31" s="38"/>
+      <c r="B31" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="44">
+      <c r="C31" s="15">
         <v>9</v>
       </c>
-      <c r="D31" s="46" t="s">
-        <v>91</v>
-      </c>
-      <c r="E31" s="24"/>
-      <c r="F31" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="G31" s="14"/>
-      <c r="H31" s="21" t="b">
+      <c r="D31" s="44" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="15"/>
+      <c r="F31" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="G31" s="22"/>
+      <c r="H31" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I31" s="26"/>
+      <c r="I31" s="36"/>
       <c r="J31" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" s="1" customFormat="1" ht="64.5" customHeight="1">
-      <c r="A32" s="40"/>
-      <c r="B32" s="27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" s="1" customFormat="1" ht="39">
+      <c r="A32" s="38"/>
+      <c r="B32" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="44">
+      <c r="C32" s="15">
         <v>4</v>
       </c>
-      <c r="D32" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E32" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>95</v>
-      </c>
-      <c r="G32" s="14"/>
-      <c r="H32" s="21" t="b">
+      <c r="D32" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="F32" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="G32" s="22"/>
+      <c r="H32" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" s="36"/>
+      <c r="J32" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="1" customFormat="1" ht="51.95">
+      <c r="A33" s="38"/>
+      <c r="B33" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" s="15"/>
+      <c r="D33" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F33" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="G33" s="22"/>
+      <c r="H33" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I32" s="26"/>
-      <c r="J32" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" s="1" customFormat="1" ht="47.25" customHeight="1">
-      <c r="A33" s="40"/>
-      <c r="B33" s="27" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" s="44">
-        <v>10</v>
-      </c>
-      <c r="D33" s="46" t="s">
-        <v>96</v>
-      </c>
-      <c r="E33" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="F33" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="G33" s="14"/>
-      <c r="H33" s="21" t="b">
+      <c r="I33" s="36"/>
+      <c r="J33" s="29"/>
+    </row>
+    <row r="34" spans="1:10" s="1" customFormat="1" ht="39">
+      <c r="A34" s="38"/>
+      <c r="B34" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="15"/>
+      <c r="D34" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="G34" s="22"/>
+      <c r="H34" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I33" s="26"/>
-      <c r="J33" s="29"/>
-    </row>
-    <row r="34" spans="1:10" s="1" customFormat="1" ht="66" customHeight="1">
-      <c r="A34" s="40"/>
-      <c r="B34" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C34" s="44"/>
-      <c r="D34" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="F34" s="36" t="s">
-        <v>99</v>
-      </c>
-      <c r="G34" s="14"/>
-      <c r="H34" s="21" t="b">
+      <c r="I34" s="16"/>
+      <c r="J34" s="29"/>
+    </row>
+    <row r="35" spans="1:10" s="1" customFormat="1" ht="120">
+      <c r="A35" s="38"/>
+      <c r="B35" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="15">
+        <v>6</v>
+      </c>
+      <c r="D35" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="G35" s="22">
+        <v>1</v>
+      </c>
+      <c r="H35" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="J35" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" s="1" customFormat="1" ht="120">
+      <c r="A36" s="38"/>
+      <c r="B36" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="15">
+        <v>6</v>
+      </c>
+      <c r="D36" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="G36" s="22">
+        <v>1</v>
+      </c>
+      <c r="H36" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="J36" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" s="1" customFormat="1" ht="65.099999999999994">
+      <c r="A37" s="38"/>
+      <c r="B37" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="15">
+        <v>7</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="G37" s="22">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37" s="16"/>
+      <c r="J37" s="29"/>
+    </row>
+    <row r="38" spans="1:10" s="1" customFormat="1" ht="75.75">
+      <c r="A38" s="38"/>
+      <c r="B38" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="15">
+        <v>8</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="G38" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="H38" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I38" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="J38" s="29"/>
+    </row>
+    <row r="39" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A39" s="38"/>
+      <c r="B39" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="15">
+        <v>3</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="G39" s="22"/>
+      <c r="H39" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I34" s="26"/>
-      <c r="J34" s="29"/>
-    </row>
-    <row r="35" spans="1:10" s="1" customFormat="1" ht="43.5" customHeight="1">
-      <c r="A35" s="40"/>
-      <c r="B35" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" s="44"/>
-      <c r="D35" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="E35" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="F35" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="G35" s="14"/>
-      <c r="H35" s="21" t="b">
+      <c r="I39" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J39" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A40" s="38"/>
+      <c r="B40" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" s="15">
+        <v>9</v>
+      </c>
+      <c r="D40" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="G40" s="22"/>
+      <c r="H40" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I35" s="16"/>
-      <c r="J35" s="29"/>
-    </row>
-    <row r="36" spans="1:10" s="1" customFormat="1" ht="91.5" customHeight="1">
-      <c r="A36" s="40"/>
-      <c r="B36" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C36" s="44">
-        <v>6</v>
-      </c>
-      <c r="D36" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="F36" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="G36" s="14">
+      <c r="I40" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="J40" s="29" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="1" customFormat="1" ht="75">
+      <c r="A41" s="38"/>
+      <c r="B41" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="15">
+        <v>3</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="G41" s="22"/>
+      <c r="H41" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="H36" s="21" t="b">
+      <c r="I41" s="16"/>
+      <c r="J41" s="34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="1" customFormat="1" ht="38.25">
+      <c r="A42" s="38"/>
+      <c r="B42" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="15">
+        <v>3</v>
+      </c>
+      <c r="D42" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="F42" s="16"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="J42" s="34"/>
+    </row>
+    <row r="43" spans="1:10" s="1" customFormat="1" ht="135">
+      <c r="A43" s="38"/>
+      <c r="B43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" s="15">
+        <v>3</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="F43" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="G43" s="22"/>
+      <c r="H43" s="43" t="b">
         <v>1</v>
-      </c>
-      <c r="I36" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="J36" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" s="1" customFormat="1" ht="101.25" customHeight="1">
-      <c r="A37" s="40"/>
-      <c r="B37" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C37" s="44">
-        <v>6</v>
-      </c>
-      <c r="D37" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="F37" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="G37" s="14">
-        <v>1</v>
-      </c>
-      <c r="H37" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="J37" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" s="1" customFormat="1" ht="95.25" customHeight="1">
-      <c r="A38" s="40"/>
-      <c r="B38" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38" s="44">
-        <v>7</v>
-      </c>
-      <c r="D38" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="F38" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" s="14"/>
-      <c r="H38" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I38" s="16"/>
-      <c r="J38" s="29"/>
-    </row>
-    <row r="39" spans="1:10" s="1" customFormat="1" ht="83.25" customHeight="1">
-      <c r="A39" s="40"/>
-      <c r="B39" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" s="44">
-        <v>8</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="E39" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="H39" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I39" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="J39" s="29"/>
-    </row>
-    <row r="40" spans="1:10" s="1" customFormat="1" ht="66.75" customHeight="1">
-      <c r="A40" s="40"/>
-      <c r="B40" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" s="44">
-        <v>3</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="E40" s="24" t="s">
-        <v>116</v>
-      </c>
-      <c r="F40" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="G40" s="14"/>
-      <c r="H40" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I40" s="16"/>
-      <c r="J40" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" s="1" customFormat="1" ht="50.25" customHeight="1">
-      <c r="A41" s="40"/>
-      <c r="B41" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41" s="44">
-        <v>9</v>
-      </c>
-      <c r="D41" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="E41" s="24" t="s">
-        <v>116</v>
-      </c>
-      <c r="F41" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="G41" s="14"/>
-      <c r="H41" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I41" s="16"/>
-      <c r="J41" s="29" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" s="1" customFormat="1" ht="83.25" customHeight="1">
-      <c r="A42" s="40"/>
-      <c r="B42" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C42" s="44">
-        <v>3</v>
-      </c>
-      <c r="D42" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="E42" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="F42" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="G42" s="14"/>
-      <c r="H42" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I42" s="16"/>
-      <c r="J42" s="34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" s="1" customFormat="1" ht="61.5" customHeight="1">
-      <c r="A43" s="40"/>
-      <c r="B43" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C43" s="44">
-        <v>3</v>
-      </c>
-      <c r="D43" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="E43" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="F43" s="16"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="21" t="b">
-        <v>0</v>
       </c>
       <c r="I43" s="16"/>
       <c r="J43" s="34"/>
     </row>
-    <row r="44" spans="1:10" s="1" customFormat="1" ht="130.5" customHeight="1">
-      <c r="A44" s="40"/>
-      <c r="B44" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C44" s="24">
-        <v>3</v>
-      </c>
-      <c r="D44" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="E44" s="24" t="s">
-        <v>125</v>
+    <row r="44" spans="1:10" s="1" customFormat="1" ht="38.25">
+      <c r="A44" s="38"/>
+      <c r="B44" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" s="15"/>
+      <c r="D44" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>137</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="G44" s="23"/>
-      <c r="H44" s="48" t="b">
-        <v>0</v>
+        <v>138</v>
+      </c>
+      <c r="G44" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="H44" s="43" t="b">
+        <v>1</v>
       </c>
       <c r="I44" s="16"/>
       <c r="J44" s="34"/>
     </row>
-    <row r="45" spans="1:10" s="1" customFormat="1" ht="47.25" customHeight="1">
-      <c r="A45" s="40"/>
-      <c r="B45" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C45" s="24"/>
-      <c r="D45" s="51" t="s">
-        <v>127</v>
-      </c>
-      <c r="E45" s="24" t="s">
-        <v>128</v>
+    <row r="45" spans="1:10" s="1" customFormat="1">
+      <c r="A45" s="38"/>
+      <c r="B45" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="15"/>
+      <c r="D45" s="69" t="s">
+        <v>140</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>141</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="G45" s="23"/>
-      <c r="H45" s="48" t="b">
+        <v>59</v>
+      </c>
+      <c r="G45" s="22"/>
+      <c r="H45" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I45" s="16"/>
+      <c r="I45" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="J45" s="34"/>
     </row>
-    <row r="46" spans="1:10" s="1" customFormat="1" ht="15.95">
-      <c r="A46" s="40"/>
-      <c r="B46" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C46" s="24"/>
-      <c r="D46" s="52" t="s">
-        <v>130</v>
-      </c>
-      <c r="E46" s="24" t="s">
-        <v>131</v>
+    <row r="46" spans="1:10" s="1" customFormat="1" ht="15.75">
+      <c r="A46" s="38"/>
+      <c r="B46" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" s="15"/>
+      <c r="D46" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="E46" s="15" t="s">
+        <v>141</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="G46" s="23"/>
-      <c r="H46" s="48" t="b">
-        <v>0</v>
+        <v>143</v>
+      </c>
+      <c r="G46" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H46" s="43" t="b">
+        <v>1</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="34"/>
     </row>
-    <row r="47" spans="1:10" s="1" customFormat="1" ht="15.95">
-      <c r="A47" s="40"/>
-      <c r="B47" s="19" t="s">
+    <row r="47" spans="1:10" s="1" customFormat="1" ht="51.95">
+      <c r="A47" s="38"/>
+      <c r="B47" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="C47" s="15"/>
+      <c r="D47" s="51" t="s">
+        <v>145</v>
+      </c>
+      <c r="E47" s="52" t="s">
+        <v>146</v>
+      </c>
+      <c r="F47" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="G47" s="22"/>
+      <c r="H47" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="J47" s="34"/>
+    </row>
+    <row r="48" spans="1:10" s="1" customFormat="1" ht="39">
+      <c r="A48" s="38"/>
+      <c r="B48" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" s="15"/>
+      <c r="D48" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="E48" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="F48" s="49" t="s">
+        <v>151</v>
+      </c>
+      <c r="G48" s="22"/>
+      <c r="H48" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="J48" s="34"/>
+    </row>
+    <row r="49" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A49" s="38"/>
+      <c r="B49" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C49" s="15"/>
+      <c r="D49" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="E49" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="F49" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="G49" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H49" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I49" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J49" s="34"/>
+    </row>
+    <row r="50" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A50" s="38"/>
+      <c r="B50" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C50" s="15"/>
+      <c r="D50" s="51" t="s">
+        <v>156</v>
+      </c>
+      <c r="E50" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="F50" s="36" t="s">
+        <v>157</v>
+      </c>
+      <c r="G50" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H50" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I50" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J50" s="34"/>
+    </row>
+    <row r="51" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A51" s="38"/>
+      <c r="B51" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="15"/>
+      <c r="D51" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="E51" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="F51" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="G51" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H51" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I51" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J51" s="34"/>
+    </row>
+    <row r="52" spans="1:10" s="1" customFormat="1" ht="30">
+      <c r="A52" s="38"/>
+      <c r="B52" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C52" s="15"/>
+      <c r="D52" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="E52" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="F52" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="G52" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H52" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I52" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J52" s="34"/>
+    </row>
+    <row r="53" spans="1:10" s="1" customFormat="1" ht="39">
+      <c r="A53" s="38"/>
+      <c r="B53" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C53" s="15"/>
+      <c r="D53" s="51" t="s">
+        <v>162</v>
+      </c>
+      <c r="E53" s="52" t="s">
+        <v>163</v>
+      </c>
+      <c r="F53" s="49" t="s">
+        <v>164</v>
+      </c>
+      <c r="G53" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="H53" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I53" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J53" s="34"/>
+    </row>
+    <row r="54" spans="1:10" s="1" customFormat="1" ht="104.1">
+      <c r="A54" s="38"/>
+      <c r="B54" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C54" s="15"/>
+      <c r="D54" s="51" t="s">
+        <v>166</v>
+      </c>
+      <c r="E54" s="52" t="s">
+        <v>167</v>
+      </c>
+      <c r="F54" s="49" t="s">
+        <v>168</v>
+      </c>
+      <c r="G54" s="22"/>
+      <c r="H54" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" s="61" t="s">
+        <v>169</v>
+      </c>
+      <c r="J54" s="34"/>
+    </row>
+    <row r="55" spans="1:10" s="1" customFormat="1" ht="45">
+      <c r="A55" s="38"/>
+      <c r="B55" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C55" s="15"/>
+      <c r="D55" s="51" t="s">
+        <v>170</v>
+      </c>
+      <c r="E55" s="52" t="s">
+        <v>167</v>
+      </c>
+      <c r="F55" s="49" t="s">
+        <v>171</v>
+      </c>
+      <c r="G55" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="H55" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I55" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J55" s="34"/>
+    </row>
+    <row r="56" spans="1:10" s="1" customFormat="1" ht="30">
+      <c r="A56" s="38"/>
+      <c r="B56" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C56" s="15"/>
+      <c r="D56" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="E56" s="52" t="s">
+        <v>167</v>
+      </c>
+      <c r="F56" s="49" t="s">
+        <v>173</v>
+      </c>
+      <c r="G56" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="H56" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I56" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="J56" s="34"/>
+    </row>
+    <row r="57" spans="1:10" s="1" customFormat="1">
+      <c r="A57" s="38"/>
+      <c r="B57" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C57" s="15">
+        <v>10</v>
+      </c>
+      <c r="D57" s="51" t="s">
+        <v>174</v>
+      </c>
+      <c r="E57" s="52" t="s">
+        <v>109</v>
+      </c>
+      <c r="F57" s="53"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" s="60" t="s">
         <v>132</v>
       </c>
-      <c r="C47" s="24"/>
-      <c r="D47" s="52" t="s">
-        <v>133</v>
-      </c>
-      <c r="E47" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="G47" s="23"/>
-      <c r="H47" s="48" t="b">
-        <v>0</v>
-      </c>
-      <c r="I47" s="16"/>
-      <c r="J47" s="34"/>
-    </row>
-    <row r="48" spans="1:10" s="1" customFormat="1" ht="63.75" customHeight="1">
-      <c r="A48" s="40"/>
-      <c r="B48" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="C48" s="44"/>
-      <c r="D48" s="53" t="s">
-        <v>136</v>
-      </c>
-      <c r="E48" s="54" t="s">
-        <v>137</v>
-      </c>
-      <c r="F48" s="51" t="s">
-        <v>138</v>
-      </c>
-      <c r="G48" s="14"/>
-      <c r="H48" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I48" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="J48" s="34"/>
-    </row>
-    <row r="49" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A49" s="40"/>
-      <c r="B49" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C49" s="44"/>
-      <c r="D49" s="53" t="s">
-        <v>140</v>
-      </c>
-      <c r="E49" s="54" t="s">
-        <v>141</v>
-      </c>
-      <c r="F49" s="51" t="s">
-        <v>142</v>
-      </c>
-      <c r="G49" s="14"/>
-      <c r="H49" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I49" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="J49" s="34"/>
-    </row>
-    <row r="50" spans="1:10" s="1" customFormat="1" ht="63.75" customHeight="1">
-      <c r="A50" s="40"/>
-      <c r="B50" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C50" s="44"/>
-      <c r="D50" s="53" t="s">
-        <v>143</v>
-      </c>
-      <c r="E50" s="54" t="s">
+      <c r="J57" s="34"/>
+    </row>
+    <row r="58" spans="1:10" s="1" customFormat="1" ht="78">
+      <c r="A58" s="38"/>
+      <c r="B58" s="47" t="s">
         <v>144</v>
       </c>
-      <c r="F50" s="51" t="s">
-        <v>145</v>
-      </c>
-      <c r="G50" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="H50" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I50" s="62" t="s">
-        <v>147</v>
-      </c>
-      <c r="J50" s="34"/>
-    </row>
-    <row r="51" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A51" s="40"/>
-      <c r="B51" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C51" s="44"/>
-      <c r="D51" s="53" t="s">
-        <v>148</v>
-      </c>
-      <c r="E51" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="F51" s="51" t="s">
-        <v>150</v>
-      </c>
-      <c r="G51" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="H51" s="21" t="b">
+      <c r="C58" s="15"/>
+      <c r="D58" s="51" t="s">
+        <v>175</v>
+      </c>
+      <c r="E58" s="52" t="s">
+        <v>176</v>
+      </c>
+      <c r="F58" s="48" t="s">
+        <v>177</v>
+      </c>
+      <c r="G58" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="H58" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I51" s="62" t="s">
-        <v>147</v>
-      </c>
-      <c r="J51" s="34"/>
-    </row>
-    <row r="52" spans="1:10" s="1" customFormat="1" ht="90.95">
-      <c r="A52" s="40"/>
-      <c r="B52" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C52" s="44"/>
-      <c r="D52" s="53" t="s">
-        <v>152</v>
-      </c>
-      <c r="E52" s="54" t="s">
-        <v>153</v>
-      </c>
-      <c r="F52" s="51" t="s">
-        <v>154</v>
-      </c>
-      <c r="G52" s="14"/>
-      <c r="H52" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I52" s="63" t="s">
-        <v>155</v>
-      </c>
-      <c r="J52" s="34"/>
-    </row>
-    <row r="53" spans="1:10" s="1" customFormat="1" ht="39">
-      <c r="A53" s="40"/>
-      <c r="B53" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C53" s="44"/>
-      <c r="D53" s="53" t="s">
-        <v>156</v>
-      </c>
-      <c r="E53" s="54" t="s">
-        <v>153</v>
-      </c>
-      <c r="F53" s="51" t="s">
-        <v>157</v>
-      </c>
-      <c r="G53" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="H53" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I53" s="62" t="s">
-        <v>147</v>
-      </c>
-      <c r="J53" s="34"/>
-    </row>
-    <row r="54" spans="1:10" s="1" customFormat="1" ht="15.95">
-      <c r="A54" s="40"/>
-      <c r="B54" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="C54" s="44">
-        <v>10</v>
-      </c>
-      <c r="D54" s="53" t="s">
-        <v>160</v>
-      </c>
-      <c r="E54" s="54" t="s">
-        <v>101</v>
-      </c>
-      <c r="F54" s="55"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="I54" s="62"/>
-      <c r="J54" s="34"/>
-    </row>
-    <row r="55" spans="1:10" s="1" customFormat="1" ht="96" customHeight="1">
-      <c r="A55" s="40"/>
-      <c r="B55" s="49" t="s">
-        <v>135</v>
-      </c>
-      <c r="C55" s="44"/>
-      <c r="D55" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="E55" s="54" t="s">
-        <v>162</v>
-      </c>
-      <c r="F55" s="50" t="s">
-        <v>163</v>
-      </c>
-      <c r="G55" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="H55" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="I55" s="62" t="s">
-        <v>147</v>
-      </c>
-      <c r="J55" s="34"/>
-    </row>
-    <row r="56" spans="1:10" s="1" customFormat="1">
-      <c r="A56" s="40"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="56"/>
-      <c r="F56" s="57"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="34"/>
-    </row>
-    <row r="57" spans="1:10" s="1" customFormat="1">
-      <c r="A57" s="40"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="8"/>
-      <c r="E57" s="58"/>
-      <c r="F57" s="59"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="8"/>
-      <c r="I57" s="8"/>
-      <c r="J57" s="34"/>
-    </row>
-    <row r="58" spans="1:10" s="1" customFormat="1" ht="18.75">
-      <c r="A58" s="40"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="65"/>
-      <c r="F58" s="60"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
+      <c r="I58" s="60" t="s">
+        <v>179</v>
+      </c>
       <c r="J58" s="34"/>
     </row>
-    <row r="59" spans="1:10" ht="18.75">
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="65"/>
-      <c r="F59" s="61"/>
-      <c r="G59" s="6"/>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6"/>
-    </row>
-    <row r="60" spans="1:10" ht="18.75">
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="65"/>
-      <c r="F60" s="61"/>
-      <c r="G60" s="6"/>
-      <c r="H60" s="6"/>
-      <c r="I60" s="6"/>
-    </row>
-    <row r="61" spans="1:10" ht="18.75">
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="65"/>
-      <c r="F61" s="61"/>
-      <c r="G61" s="6"/>
-      <c r="H61" s="6"/>
-      <c r="I61" s="6"/>
-    </row>
-    <row r="62" spans="1:10" ht="18.75">
+    <row r="59" spans="1:10" s="1" customFormat="1">
+      <c r="A59" s="38"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="54"/>
+      <c r="F59" s="55"/>
+      <c r="G59" s="65"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="34"/>
+    </row>
+    <row r="60" spans="1:10" s="1" customFormat="1">
+      <c r="A60" s="38"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="57"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8"/>
+      <c r="J60" s="34"/>
+    </row>
+    <row r="61" spans="1:10" s="1" customFormat="1" ht="18.600000000000001">
+      <c r="A61" s="38"/>
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="68"/>
+      <c r="F61" s="58"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4"/>
+      <c r="J61" s="34"/>
+    </row>
+    <row r="62" spans="1:10" ht="18.600000000000001">
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
       <c r="D62" s="6"/>
-      <c r="E62" s="65"/>
-      <c r="F62" s="61"/>
-      <c r="G62" s="6"/>
+      <c r="E62" s="68"/>
+      <c r="F62" s="59"/>
+      <c r="G62" s="67"/>
       <c r="H62" s="6"/>
       <c r="I62" s="6"/>
     </row>
-    <row r="63" spans="1:10" ht="18.75">
+    <row r="63" spans="1:10" ht="18.600000000000001">
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
       <c r="D63" s="6"/>
-      <c r="E63" s="65"/>
-      <c r="F63" s="61"/>
-      <c r="G63" s="6"/>
+      <c r="E63" s="68"/>
+      <c r="F63" s="59"/>
+      <c r="G63" s="67"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
     </row>
-    <row r="64" spans="1:10" ht="18.75">
+    <row r="64" spans="1:10" ht="18.600000000000001">
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
       <c r="D64" s="6"/>
-      <c r="E64" s="65"/>
-      <c r="F64" s="61"/>
-      <c r="G64" s="6"/>
+      <c r="E64" s="68"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="67"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6"/>
     </row>
-    <row r="65" spans="2:9" ht="18.75">
+    <row r="65" spans="2:9" ht="18.600000000000001">
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="6"/>
-      <c r="G65" s="6"/>
+      <c r="E65" s="68"/>
+      <c r="F65" s="59"/>
+      <c r="G65" s="67"/>
       <c r="H65" s="6"/>
       <c r="I65" s="6"/>
     </row>
-    <row r="66" spans="2:9" ht="18.75">
+    <row r="66" spans="2:9" ht="18.600000000000001">
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
       <c r="D66" s="6"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="6"/>
-      <c r="G66" s="6"/>
+      <c r="E66" s="68"/>
+      <c r="F66" s="59"/>
+      <c r="G66" s="67"/>
       <c r="H66" s="6"/>
       <c r="I66" s="6"/>
     </row>
+    <row r="67" spans="2:9" ht="18.600000000000001">
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="68"/>
+      <c r="F67" s="59"/>
+      <c r="G67" s="67"/>
+      <c r="H67" s="6"/>
+      <c r="I67" s="6"/>
+    </row>
+    <row r="68" spans="2:9" ht="18.600000000000001">
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
+      <c r="H68" s="6"/>
+      <c r="I68" s="6"/>
+    </row>
+    <row r="69" spans="2:9" ht="18.600000000000001">
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J55" xr:uid="{07127F19-9F63-3B48-ABE6-8FC4ADCB9798}"/>
+  <autoFilter ref="A3:J58" xr:uid="{07127F19-9F63-3B48-ABE6-8FC4ADCB9798}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f0974581-4bbf-443e-902f-14073e9fb4f6" xsi:nil="true"/>
-    <Preview xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-    <Manualcategory xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006958AF0A0D18DD46AA2F05B0B7FB2051" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7cc4835c91b31b9b519dddda0e0127ea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8743faf2-653b-47e5-938e-a3c18a0572b2" xmlns:ns3="65bb3d2a-ea9e-471d-8113-08ea35fd4d0a" xmlns:ns4="f0974581-4bbf-443e-902f-14073e9fb4f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b07298893fe1b0d1a251a8914f437576" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="8743faf2-653b-47e5-938e-a3c18a0572b2"/>
@@ -3587,6 +3874,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f0974581-4bbf-443e-902f-14073e9fb4f6" xsi:nil="true"/>
+    <Preview xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+    <Manualcategory xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3597,11 +3898,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58C97B2E-9E09-49C0-88E7-D25203A87982}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{113860E7-0903-4CD1-86F2-CB3C963E0E6D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A4CDDC2-C00E-4008-8D54-8631B32BE295}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58C97B2E-9E09-49C0-88E7-D25203A87982}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Uusi Excel, parserikorjaukset, esteet ja toiveet päivitetty
- Parseri: puolipiste-erotin, yhdysviiva-sukunimet, mixed-case korjaus
- Domain-prefiksit: Core, B2B Core, Display team lisätty
- Aliakset: Laura KAngas, Jonne Ansama, ym.
- Exclude: "ei dep syncciin" lisätty (14 sessiota pois)
- Esteet: 14 henkilölle ke 9:30-10:30
- Toive: natiivi-sessio ei ti klo 12 jälkeen
- 41 sessiota, 119 henkilöä, 17 konfliktiä

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
+++ b/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sanoma.sharepoint.com/sites/B2BGeneral667/Shared Documents/General/B2B (STEP) Cross-Domain Public/Seasonal Planning Process/2026_S3 materials/Dependency Synchronization Days/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEE73A60-7162-4EA3-93BD-01488BFDAD5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{81731090-F27C-4A31-A725-A9EC2F8C0110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="18980" xr2:uid="{86D0FE88-11BB-614D-BBC1-5CCA99757B8D}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="181">
   <si>
     <t>S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08</t>
   </si>
@@ -100,7 +100,7 @@
     <t>Jaana Tynys</t>
   </si>
   <si>
-    <t>Filip Homberg, Jaana Tanskanen, Jaakko Kuivalainen, Mikko Neva</t>
+    <t>Filip Holmberg, Jaana Tanskanen, Jaakko Kuivalainen, Mikko Neva</t>
   </si>
   <si>
     <t>Oma e2e arvotiimi tai ohjausryhmä (?) - input:ksi brief</t>
@@ -141,11 +141,13 @@
     <t xml:space="preserve">
 Heidi Falenius
 Satu Raatikainen
-Leena Koskinen
+Leena Koskinen, Anna Schoschkoff
 DSE&amp;A: Vesa Lindqvist, Tanja Kaikkonen
 Jaana Tanskanen
 DG: Tuuli Rikama, Tuukka Antikainen
-Print: Päivi Vaittinen
+Print: Päivi Vaittinen, Maria Ryssy
+TV &amp; audio: Pia Viinikainen
+Myynti: Tiina Kosonen
 </t>
   </si>
   <si>
@@ -399,13 +401,34 @@
     <t>- Avauksen rooli: Terhi+Ossi?</t>
   </si>
   <si>
-    <t>ei suunnittelua</t>
+    <t xml:space="preserve">Ei dep syncciin </t>
   </si>
   <si>
     <t>DSE Prio 10: Yhteinen kaupallinen johtamismalli/RevOps: Yhteisen kaupallisen johtamismallin luonti ja käyttöönotto pienemmän asiakassegmentin osalta (RevOps) ja markkinoinnin yhteistyön selkeyttäminen osana kompetenssityötä</t>
   </si>
   <si>
     <t xml:space="preserve">Työryhmän startti: Maiju Häkkinen, Perttu Rekola, Tiina Kosonen, Vesa Lindqvist, CX xxx, markkinointi xx, </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ei dep syncciin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, etenee erillisellä aikataululla</t>
+    </r>
   </si>
   <si>
     <t>DSE Prio 10: Yhteinen kaupallinen johtamismalli: Kehitämme prospektointia ja Skoutti –pelinrakentajaa.</t>
@@ -456,7 +479,25 @@
 Jaana Tanskanen</t>
   </si>
   <si>
-    <t>25.8 klo 14-15 (Leena jo buukannut)</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ei dep syncciin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.25.8 klo 14-15 (Leena jo buukannut)</t>
+    </r>
   </si>
   <si>
     <t>Sales KPI: myynnin raportoinnin &amp; dashboard datojen haasteet ratkottava laittamalla kuntoon perusta datatuotteistuksen osalta jotta datakehitys tehdään agenttilähtöiseksi, ei raporttilähtöisesti. Edellyttää uudenlaista osaamista ja focusta tiimiin.
@@ -479,7 +520,25 @@
     <t>Janne Nurmisto,  Tuomo Sinkkonen, Lotta Monten, Minna Kruhse, Riku Talvitie, Leena Koskinen, Tiina Kosonen, Hanna Jalonen</t>
   </si>
   <si>
-    <t>Tämä ti 13-14 Product Sales tiimiksen aikaan (buukattu)</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ei dep syncciin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Tämä ti 13-14 Product Sales tiimiksen aikaan (buukattu)</t>
+    </r>
   </si>
   <si>
     <t>Tuloksellisuus. Tavoite ja mittarimallin seuraavat vaiheet &amp; vaikutukset eri domaineille (odotukset painottuen S1, mutta domainien odotetaan arvioivan ja huomioivan vaikutuksia jo S3 nykyisessä tekemisessä)</t>
@@ -524,7 +583,7 @@
     <t>Filip Holmberg, Jaana Tanskanen, Jonne Ansamaa, Nea Särkikoski, Niko-Petteri Varho</t>
   </si>
   <si>
-    <t>Ei dep syncciin. Toive, että 1vk myöhemmin</t>
+    <t>Toive, että 1vk myöhemmin</t>
   </si>
   <si>
     <t>Discovery: kasvupalvelun asiakkaiden mainosdatan rikastaminen tulosten parantamiseksi; vaihtoehtojen kartoitus ja pilotointi. Datan parannus melko domainin sisäinen työ, mutta pitää huomioida raportointi ja datayhteys näkökulmasta</t>
@@ -533,7 +592,25 @@
     <t>John Kronström, TBD</t>
   </si>
   <si>
-    <t>Ei dep syncciin. Toive, että 2vk myöhemmin</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Ei dep syncciin.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Toive, että 2vk myöhemmin</t>
+    </r>
   </si>
   <si>
     <t>Kasvuraportin kehitystyö, jatkokehitys (pienkehitys)</t>
@@ -552,17 +629,23 @@
 DG: Tuuli Rikama, Tuukka Antikainen</t>
   </si>
   <si>
-    <t>B2B Prio 8, MSS PRIO 5: Medialle natiivimainonnalla parempi kuluttajakokemus sekä parempi mainonnan vaikuttavuus sekä yield
-Natiivistrategian rakentaminen: natiivin julkaisujärjestelmän evaluaatio</t>
-  </si>
-  <si>
-    <t>Ria Vaahto &amp; Petra Saikku</t>
-  </si>
-  <si>
-    <t>MSS Media solutions natiivi: Ria Vaahto &amp; Petra Saikku
+    <t xml:space="preserve">B2B Prio 8, MSS PRIO 5: Medialle natiivimainonnalla parempi vaikuttavuus sekä yield
+</t>
+  </si>
+  <si>
+    <t>Ria Vaahto</t>
+  </si>
+  <si>
+    <t>MSS Media solutions natiivi: Ria Vaahto, Petra Saikku
 DG: Johannes Hocksell, Jaakko Kuivalainen, Jonne Ansamaa
 N&amp;F: Timo Rinne, Anssi Hämäläinen, Teemu Hauhia, Sanna Wirkkala
 Yield: Tuukka Antikainen, Aki Salonen</t>
+  </si>
+  <si>
+    <t>1,5h</t>
+  </si>
+  <si>
+    <t>Ei ti klo 12 jälkeen, jos mahdollista</t>
   </si>
   <si>
     <t>Ratkaisunrakentaja visio --&gt; ei riippuvuussuunnitteluun,  Mikko N. kontaktoi erikseen tarpeiden keskustelua
@@ -823,6 +906,9 @@
 Sami Luutikivi</t>
   </si>
   <si>
+    <t>2h</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -845,7 +931,7 @@
     </r>
   </si>
   <si>
-    <t>Ei dep syncciin</t>
+    <t>Ad Manager: Toni Törnqvist, Anniina Hautala; Display team: Emmy Ramsay; Core: Heidi Falenius; CPR: Jonne Ansama; Performance Products: Hannu Häikiö, Johannes Hocksell</t>
   </si>
   <si>
     <r>
@@ -959,9 +1045,6 @@
 Sales &amp; Marketing​</t>
   </si>
   <si>
-    <t>Ei pidetä omaa palaveria</t>
-  </si>
-  <si>
     <t>Skaalautuvat operatiiviset hoitomallit asiakasryhmittäin​</t>
   </si>
   <si>
@@ -996,9 +1079,6 @@
       <t xml:space="preserve"> (60 min)
 Panu Hyryläinen, Annika Palm, Joonas Imeläinen, Anu Linden, Pia Viinikainen, Heidi Falenius, Juho Pöyhönen, Antero Karttunen</t>
     </r>
-  </si>
-  <si>
-    <t>tulee dep.sync</t>
   </si>
   <si>
     <t>AV  Maestro, meeting 2</t>
@@ -1097,9 +1177,6 @@
 DSE Heidi Falenius</t>
   </si>
   <si>
-    <t>ei tarvita palaveria, ei dep syncciin</t>
-  </si>
-  <si>
     <t>TV Beat, meeting 1</t>
   </si>
   <si>
@@ -1115,6 +1192,9 @@
   </si>
   <si>
     <t>SMF tieto-omaisuuden (”data”) hallinta ja kehitys B2B:n näkökulmasta. Aloitetaan natiivin tukemisesta.​</t>
+  </si>
+  <si>
+    <t>Ei dep syncciin</t>
   </si>
   <si>
     <t xml:space="preserve">Raportointi tarpeet S3:selle. </t>
@@ -1129,16 +1209,13 @@
   </si>
   <si>
     <t>3 h</t>
-  </si>
-  <si>
-    <t>dep.sync</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1326,6 +1403,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1421,7 +1504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1605,9 +1688,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1638,6 +1718,21 @@
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2064,7 +2159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="38.25">
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="25.5">
       <c r="A4" s="38"/>
       <c r="B4" s="12" t="s">
         <v>10</v>
@@ -2090,7 +2185,7 @@
       </c>
       <c r="J4" s="34"/>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="165">
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="138.75">
       <c r="A5" s="38"/>
       <c r="B5" s="42" t="s">
         <v>15</v>
@@ -2098,7 +2193,7 @@
       <c r="C5" s="14">
         <v>2</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="28" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="23" t="s">
@@ -2111,7 +2206,7 @@
       <c r="H5" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I5" s="64"/>
+      <c r="I5" s="63"/>
       <c r="J5" s="34"/>
     </row>
     <row r="6" spans="1:10" s="1" customFormat="1" ht="128.1" customHeight="1">
@@ -2137,7 +2232,7 @@
       <c r="H6" s="33" t="b">
         <v>1</v>
       </c>
-      <c r="I6" s="64"/>
+      <c r="I6" s="63"/>
       <c r="J6" s="34"/>
     </row>
     <row r="7" spans="1:10" s="1" customFormat="1" ht="77.25">
@@ -2161,7 +2256,7 @@
       <c r="H7" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="64" t="s">
+      <c r="I7" s="63" t="s">
         <v>26</v>
       </c>
       <c r="J7" s="34"/>
@@ -2187,8 +2282,8 @@
       <c r="H8" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="64"/>
-      <c r="J8" s="70"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="69"/>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="99" customHeight="1">
       <c r="A9" s="38"/>
@@ -2210,7 +2305,7 @@
       <c r="G9" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="71" t="b">
+      <c r="H9" s="70" t="b">
         <v>1</v>
       </c>
       <c r="I9" s="16"/>
@@ -2316,7 +2411,7 @@
       <c r="I13" s="16"/>
       <c r="J13" s="34"/>
     </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="30">
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="25.5">
       <c r="A14" s="38"/>
       <c r="B14" s="19" t="s">
         <v>10</v>
@@ -2335,14 +2430,14 @@
       <c r="H14" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I14" s="16" t="s">
+      <c r="I14" s="71" t="s">
         <v>50</v>
       </c>
       <c r="J14" s="34" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="30">
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="25.5">
       <c r="A15" s="38"/>
       <c r="B15" s="19" t="s">
         <v>10</v>
@@ -2361,7 +2456,9 @@
       <c r="H15" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="I15" s="27"/>
+      <c r="I15" s="72" t="s">
+        <v>53</v>
+      </c>
       <c r="J15" s="34" t="s">
         <v>42</v>
       </c>
@@ -2375,13 +2472,13 @@
         <v>10</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G16" s="22"/>
       <c r="H16" s="33" t="b">
@@ -2399,13 +2496,13 @@
         <v>4</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G17" s="22"/>
       <c r="H17" s="43" t="b">
@@ -2420,16 +2517,16 @@
         <v>15</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G18" s="22"/>
       <c r="H18" s="33" t="b">
@@ -2438,29 +2535,29 @@
       <c r="I18" s="16"/>
       <c r="J18" s="34"/>
     </row>
-    <row r="19" spans="1:10" s="1" customFormat="1" ht="51.95">
+    <row r="19" spans="1:10" s="1" customFormat="1" ht="50.25">
       <c r="A19" s="38"/>
       <c r="B19" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="62" t="s">
-        <v>59</v>
+      <c r="C19" s="61" t="s">
+        <v>60</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G19" s="22"/>
       <c r="H19" s="33" t="b">
         <v>1</v>
       </c>
-      <c r="I19" s="16" t="s">
-        <v>65</v>
+      <c r="I19" s="24" t="s">
+        <v>66</v>
       </c>
       <c r="J19" s="34"/>
     </row>
@@ -2473,13 +2570,13 @@
         <v>31</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G20" s="22"/>
       <c r="H20" s="33" t="b">
@@ -2490,7 +2587,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:10" s="1" customFormat="1" ht="51.95">
+    <row r="21" spans="1:10" s="1" customFormat="1" ht="38.25">
       <c r="A21" s="38"/>
       <c r="B21" s="19" t="s">
         <v>15</v>
@@ -2499,13 +2596,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G21" s="22">
         <v>1</v>
@@ -2513,8 +2610,8 @@
       <c r="H21" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I21" s="16" t="s">
-        <v>72</v>
+      <c r="I21" s="24" t="s">
+        <v>73</v>
       </c>
       <c r="J21" s="34" t="s">
         <v>42</v>
@@ -2529,13 +2626,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G22" s="22">
         <v>1</v>
@@ -2555,16 +2652,16 @@
         <v>1</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H23" s="43" t="b">
         <v>1</v>
@@ -2581,13 +2678,13 @@
         <v>1</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G24" s="22">
         <v>1</v>
@@ -2596,7 +2693,7 @@
         <v>1</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J24" s="34"/>
     </row>
@@ -2608,14 +2705,14 @@
       <c r="C25" s="23">
         <v>9</v>
       </c>
-      <c r="D25" s="63" t="s">
-        <v>82</v>
+      <c r="D25" s="62" t="s">
+        <v>83</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G25" s="22"/>
       <c r="H25" s="43" t="b">
@@ -2633,20 +2730,20 @@
         <v>9</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G26" s="22"/>
       <c r="H26" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J26" s="34"/>
     </row>
@@ -2659,20 +2756,20 @@
         <v>9</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G27" s="22"/>
       <c r="H27" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I27" s="16" t="s">
-        <v>90</v>
+      <c r="I27" s="24" t="s">
+        <v>91</v>
       </c>
       <c r="J27" s="34"/>
     </row>
@@ -2684,21 +2781,21 @@
       <c r="C28" s="23">
         <v>9</v>
       </c>
-      <c r="D28" s="63" t="s">
-        <v>91</v>
+      <c r="D28" s="62" t="s">
+        <v>92</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G28" s="22"/>
       <c r="H28" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I28" s="16" t="s">
-        <v>93</v>
+      <c r="I28" s="71" t="s">
+        <v>94</v>
       </c>
       <c r="J28" s="34" t="s">
         <v>42</v>
@@ -2712,14 +2809,14 @@
       <c r="C29" s="23">
         <v>9</v>
       </c>
-      <c r="D29" s="63" t="s">
-        <v>94</v>
+      <c r="D29" s="62" t="s">
+        <v>95</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G29" s="22"/>
       <c r="H29" s="43" t="b">
@@ -2728,7 +2825,7 @@
       <c r="I29" s="16"/>
       <c r="J29" s="34"/>
     </row>
-    <row r="30" spans="1:10" s="1" customFormat="1" ht="51.95">
+    <row r="30" spans="1:10" s="1" customFormat="1" ht="65.25" customHeight="1">
       <c r="A30" s="38"/>
       <c r="B30" s="21" t="s">
         <v>30</v>
@@ -2737,19 +2834,23 @@
         <v>5</v>
       </c>
       <c r="D30" s="24" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F30" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="G30" s="22"/>
+        <v>99</v>
+      </c>
+      <c r="G30" s="22" t="s">
+        <v>100</v>
+      </c>
       <c r="H30" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I30" s="36"/>
+      <c r="I30" s="36" t="s">
+        <v>101</v>
+      </c>
       <c r="J30" s="29"/>
     </row>
     <row r="31" spans="1:10" s="1" customFormat="1" ht="39">
@@ -2761,22 +2862,24 @@
         <v>9</v>
       </c>
       <c r="D31" s="44" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E31" s="15"/>
       <c r="F31" s="25" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G31" s="22"/>
       <c r="H31" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I31" s="36"/>
+      <c r="I31" s="73" t="s">
+        <v>50</v>
+      </c>
       <c r="J31" s="29" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="32" spans="1:10" s="1" customFormat="1" ht="25.5">
       <c r="A32" s="38"/>
       <c r="B32" s="26" t="s">
         <v>10</v>
@@ -2785,15 +2888,17 @@
         <v>4</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F32" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="G32" s="22"/>
+        <v>106</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>35</v>
+      </c>
       <c r="H32" s="43" t="b">
         <v>1</v>
       </c>
@@ -2805,17 +2910,17 @@
     <row r="33" spans="1:10" s="1" customFormat="1" ht="51.95">
       <c r="A33" s="38"/>
       <c r="B33" s="26" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C33" s="15"/>
       <c r="D33" s="24" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F33" s="25" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G33" s="22"/>
       <c r="H33" s="43" t="b">
@@ -2827,17 +2932,17 @@
     <row r="34" spans="1:10" s="1" customFormat="1" ht="39">
       <c r="A34" s="38"/>
       <c r="B34" s="26" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C34" s="15"/>
       <c r="D34" s="16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G34" s="22"/>
       <c r="H34" s="43" t="b">
@@ -2855,13 +2960,13 @@
         <v>6</v>
       </c>
       <c r="D35" s="28" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G35" s="22">
         <v>1</v>
@@ -2870,7 +2975,7 @@
         <v>1</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="J35" s="29" t="s">
         <v>42</v>
@@ -2885,13 +2990,13 @@
         <v>6</v>
       </c>
       <c r="D36" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="E36" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>112</v>
-      </c>
       <c r="F36" s="13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G36" s="22">
         <v>1</v>
@@ -2900,7 +3005,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="J36" s="29" t="s">
         <v>42</v>
@@ -2915,13 +3020,13 @@
         <v>7</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G37" s="22">
         <v>1.5</v>
@@ -2941,22 +3046,22 @@
         <v>8</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="H38" s="43" t="b">
         <v>1</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="J38" s="29"/>
     </row>
@@ -2969,13 +3074,13 @@
         <v>3</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G39" s="22"/>
       <c r="H39" s="43" t="b">
@@ -2997,13 +3102,13 @@
         <v>9</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G40" s="22"/>
       <c r="H40" s="43" t="b">
@@ -3016,7 +3121,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="1" customFormat="1" ht="75">
+    <row r="41" spans="1:10" s="1" customFormat="1" ht="63">
       <c r="A41" s="38"/>
       <c r="B41" s="21" t="s">
         <v>19</v>
@@ -3025,15 +3130,17 @@
         <v>3</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="G41" s="22"/>
+        <v>133</v>
+      </c>
+      <c r="G41" s="22" t="s">
+        <v>134</v>
+      </c>
       <c r="H41" s="43" t="b">
         <v>1</v>
       </c>
@@ -3051,19 +3158,21 @@
         <v>3</v>
       </c>
       <c r="D42" s="28" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="F42" s="16"/>
-      <c r="G42" s="22"/>
+        <v>132</v>
+      </c>
+      <c r="F42" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="G42" s="22" t="s">
+        <v>35</v>
+      </c>
       <c r="H42" s="43" t="b">
-        <v>0</v>
-      </c>
-      <c r="I42" s="16" t="s">
-        <v>132</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I42" s="16"/>
       <c r="J42" s="34"/>
     </row>
     <row r="43" spans="1:10" s="1" customFormat="1" ht="135">
@@ -3075,13 +3184,13 @@
         <v>3</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="G43" s="22"/>
       <c r="H43" s="43" t="b">
@@ -3097,16 +3206,16 @@
       </c>
       <c r="C44" s="15"/>
       <c r="D44" s="49" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H44" s="43" t="b">
         <v>1</v>
@@ -3120,20 +3229,20 @@
         <v>19</v>
       </c>
       <c r="C45" s="15"/>
-      <c r="D45" s="69" t="s">
-        <v>140</v>
+      <c r="D45" s="68" t="s">
+        <v>144</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G45" s="22"/>
       <c r="H45" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I45" s="16" t="s">
+      <c r="I45" s="71" t="s">
         <v>50</v>
       </c>
       <c r="J45" s="34"/>
@@ -3145,13 +3254,13 @@
       </c>
       <c r="C46" s="15"/>
       <c r="D46" s="50" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="G46" s="22" t="s">
         <v>35</v>
@@ -3165,65 +3274,65 @@
     <row r="47" spans="1:10" s="1" customFormat="1" ht="51.95">
       <c r="A47" s="38"/>
       <c r="B47" s="21" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C47" s="15"/>
       <c r="D47" s="51" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E47" s="52" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F47" s="49" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="G47" s="22"/>
       <c r="H47" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I47" s="16" t="s">
-        <v>148</v>
+      <c r="I47" s="71" t="s">
+        <v>50</v>
       </c>
       <c r="J47" s="34"/>
     </row>
     <row r="48" spans="1:10" s="1" customFormat="1" ht="39">
       <c r="A48" s="38"/>
       <c r="B48" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C48" s="15"/>
       <c r="D48" s="51" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E48" s="52" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F48" s="49" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G48" s="22"/>
       <c r="H48" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I48" s="16" t="s">
-        <v>148</v>
+      <c r="I48" s="71" t="s">
+        <v>50</v>
       </c>
       <c r="J48" s="34"/>
     </row>
     <row r="49" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A49" s="38"/>
       <c r="B49" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C49" s="15"/>
       <c r="D49" s="51" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E49" s="52" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G49" s="22" t="s">
         <v>35</v>
@@ -3231,25 +3340,23 @@
       <c r="H49" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I49" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I49" s="60"/>
       <c r="J49" s="34"/>
     </row>
     <row r="50" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A50" s="38"/>
       <c r="B50" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C50" s="15"/>
       <c r="D50" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="E50" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="E50" s="52" t="s">
-        <v>153</v>
-      </c>
       <c r="F50" s="36" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G50" s="22" t="s">
         <v>35</v>
@@ -3257,25 +3364,23 @@
       <c r="H50" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I50" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I50" s="60"/>
       <c r="J50" s="34"/>
     </row>
     <row r="51" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A51" s="38"/>
       <c r="B51" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C51" s="15"/>
       <c r="D51" s="51" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E51" s="52" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G51" s="22" t="s">
         <v>35</v>
@@ -3283,101 +3388,95 @@
       <c r="H51" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I51" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I51" s="60"/>
       <c r="J51" s="34"/>
     </row>
     <row r="52" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A52" s="38"/>
       <c r="B52" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C52" s="15"/>
       <c r="D52" s="51" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E52" s="52" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H52" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I52" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I52" s="60"/>
       <c r="J52" s="34"/>
     </row>
     <row r="53" spans="1:10" s="1" customFormat="1" ht="39">
       <c r="A53" s="38"/>
       <c r="B53" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C53" s="15"/>
       <c r="D53" s="51" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E53" s="52" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F53" s="49" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H53" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I53" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I53" s="60"/>
       <c r="J53" s="34"/>
     </row>
     <row r="54" spans="1:10" s="1" customFormat="1" ht="104.1">
       <c r="A54" s="38"/>
       <c r="B54" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C54" s="15"/>
       <c r="D54" s="51" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E54" s="52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F54" s="49" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G54" s="22"/>
       <c r="H54" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I54" s="61" t="s">
-        <v>169</v>
+      <c r="I54" s="75" t="s">
+        <v>50</v>
       </c>
       <c r="J54" s="34"/>
     </row>
     <row r="55" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A55" s="38"/>
       <c r="B55" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C55" s="15"/>
       <c r="D55" s="51" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E55" s="52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F55" s="49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G55" s="22" t="s">
         <v>35</v>
@@ -3385,85 +3484,79 @@
       <c r="H55" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I55" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I55" s="60"/>
       <c r="J55" s="34"/>
     </row>
     <row r="56" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A56" s="38"/>
       <c r="B56" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C56" s="15"/>
       <c r="D56" s="51" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E56" s="52" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F56" s="49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H56" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I56" s="60" t="s">
-        <v>155</v>
-      </c>
+      <c r="I56" s="60"/>
       <c r="J56" s="34"/>
     </row>
     <row r="57" spans="1:10" s="1" customFormat="1">
       <c r="A57" s="38"/>
       <c r="B57" s="12" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C57" s="15">
         <v>10</v>
       </c>
       <c r="D57" s="51" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E57" s="52" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F57" s="53"/>
       <c r="G57" s="22"/>
       <c r="H57" s="43" t="b">
         <v>0</v>
       </c>
-      <c r="I57" s="60" t="s">
-        <v>132</v>
+      <c r="I57" s="74" t="s">
+        <v>176</v>
       </c>
       <c r="J57" s="34"/>
     </row>
     <row r="58" spans="1:10" s="1" customFormat="1" ht="78">
       <c r="A58" s="38"/>
       <c r="B58" s="47" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C58" s="15"/>
       <c r="D58" s="51" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E58" s="52" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F58" s="48" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H58" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="I58" s="60" t="s">
-        <v>179</v>
-      </c>
+      <c r="I58" s="60"/>
       <c r="J58" s="34"/>
     </row>
     <row r="59" spans="1:10" s="1" customFormat="1">
@@ -3473,7 +3566,7 @@
       <c r="D59" s="11"/>
       <c r="E59" s="54"/>
       <c r="F59" s="55"/>
-      <c r="G59" s="65"/>
+      <c r="G59" s="64"/>
       <c r="H59" s="11"/>
       <c r="I59" s="11"/>
       <c r="J59" s="34"/>
@@ -3494,9 +3587,9 @@
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="4"/>
-      <c r="E61" s="68"/>
+      <c r="E61" s="67"/>
       <c r="F61" s="58"/>
-      <c r="G61" s="66"/>
+      <c r="G61" s="65"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="34"/>
@@ -3505,9 +3598,9 @@
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
       <c r="D62" s="6"/>
-      <c r="E62" s="68"/>
+      <c r="E62" s="67"/>
       <c r="F62" s="59"/>
-      <c r="G62" s="67"/>
+      <c r="G62" s="66"/>
       <c r="H62" s="6"/>
       <c r="I62" s="6"/>
     </row>
@@ -3515,9 +3608,9 @@
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
       <c r="D63" s="6"/>
-      <c r="E63" s="68"/>
+      <c r="E63" s="67"/>
       <c r="F63" s="59"/>
-      <c r="G63" s="67"/>
+      <c r="G63" s="66"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
     </row>
@@ -3525,9 +3618,9 @@
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
       <c r="D64" s="6"/>
-      <c r="E64" s="68"/>
+      <c r="E64" s="67"/>
       <c r="F64" s="59"/>
-      <c r="G64" s="67"/>
+      <c r="G64" s="66"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6"/>
     </row>
@@ -3535,9 +3628,9 @@
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
-      <c r="E65" s="68"/>
+      <c r="E65" s="67"/>
       <c r="F65" s="59"/>
-      <c r="G65" s="67"/>
+      <c r="G65" s="66"/>
       <c r="H65" s="6"/>
       <c r="I65" s="6"/>
     </row>
@@ -3545,9 +3638,9 @@
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
       <c r="D66" s="6"/>
-      <c r="E66" s="68"/>
+      <c r="E66" s="67"/>
       <c r="F66" s="59"/>
-      <c r="G66" s="67"/>
+      <c r="G66" s="66"/>
       <c r="H66" s="6"/>
       <c r="I66" s="6"/>
     </row>
@@ -3555,9 +3648,9 @@
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
       <c r="D67" s="6"/>
-      <c r="E67" s="68"/>
+      <c r="E67" s="67"/>
       <c r="F67" s="59"/>
-      <c r="G67" s="67"/>
+      <c r="G67" s="66"/>
       <c r="H67" s="6"/>
       <c r="I67" s="6"/>
     </row>
@@ -3589,6 +3682,29 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f0974581-4bbf-443e-902f-14073e9fb4f6" xsi:nil="true"/>
+    <Preview xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+    <Manualcategory xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006958AF0A0D18DD46AA2F05B0B7FB2051" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7cc4835c91b31b9b519dddda0e0127ea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8743faf2-653b-47e5-938e-a3c18a0572b2" xmlns:ns3="65bb3d2a-ea9e-471d-8113-08ea35fd4d0a" xmlns:ns4="f0974581-4bbf-443e-902f-14073e9fb4f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b07298893fe1b0d1a251a8914f437576" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="8743faf2-653b-47e5-938e-a3c18a0572b2"/>
@@ -3874,37 +3990,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f0974581-4bbf-443e-902f-14073e9fb4f6" xsi:nil="true"/>
-    <Preview xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-    <Manualcategory xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="8743faf2-653b-47e5-938e-a3c18a0572b2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{113860E7-0903-4CD1-86F2-CB3C963E0E6D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58C97B2E-9E09-49C0-88E7-D25203A87982}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58C97B2E-9E09-49C0-88E7-D25203A87982}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE028EC4-4BAF-4D78-8C7F-C3E8970CA932}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE028EC4-4BAF-4D78-8C7F-C3E8970CA932}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{113860E7-0903-4CD1-86F2-CB3C963E0E6D}"/>
 </file>
</xml_diff>

<commit_message>
Uusin Excel, nimiparsinnan korjaukset, omistaja-overlap-esto, lukituskorjaus
- Uusin Excel-versio (17.08), 41 sessiota, 123 henkilöä
- Parseri: "ja"/"and" nimitunnistus, sulkunimien ohitus info-kentän perusteella
- Parseri: "ei tarvita" ei enää sulje pois sessioita joissa viitataan osallistujiin
- Parseri: Janne Mikkola → Mikkonen alias, oletustiedosto päivitetty
- Scheduler: omistajan päällekkäisyys kova esto (ei voi fasilitoida kahdessa)
- UI: lukittujen sessioiden säilytys uudelleenaikataulutuksessa (browser-puoli)
- Janne Eräsen este ma 13-14, Satu Raatikaisen sessio-toive ma/ti
- internalOnly-kentän case-insensitive tarkistus

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
+++ b/data/S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08 (1).xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sanoma.sharepoint.com/sites/B2BGeneral667/Shared Documents/General/B2B (STEP) Cross-Domain Public/Seasonal Planning Process/2026_S3 materials/Dependency Synchronization Days/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81731090-F27C-4A31-A725-A9EC2F8C0110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15CE3B47-B217-44F5-9F71-B6F8C7A88138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="30240" windowHeight="18980" xr2:uid="{86D0FE88-11BB-614D-BBC1-5CCA99757B8D}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21020" xr2:uid="{86D0FE88-11BB-614D-BBC1-5CCA99757B8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Synccipaltsu" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">Synccipaltsu!$A$3:$J$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Synccipaltsu!$A$3:$J$58</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="181">
   <si>
     <t>S3Y26 Teknologiakehityksen ja arkkitehtuurien synkronisointipalaveri 17.08</t>
   </si>
@@ -138,16 +137,19 @@
     <t>Satu Raatikainen</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Heidi Falenius
-Satu Raatikainen
-Leena Koskinen, Anna Schoschkoff
+    <t xml:space="preserve">Heidi Falenius
+Vaalien projektipäällikkö: Satu Raatikainen
+Kaupallinen tavoite &amp; myynti: Konsta Raussi ja Tiina Kosonen
+Markkinointi: Leena Koskinen, Anna Schoschkoff
 DSE&amp;A: Vesa Lindqvist, Tanja Kaikkonen
 Jaana Tanskanen
 DG: Tuuli Rikama, Tuukka Antikainen
 Print: Päivi Vaittinen, Maria Ryssy
 TV &amp; audio: Pia Viinikainen
-Myynti: Tiina Kosonen
+Natiivi: Ria Vaahto
+Aineistotuotannot: Suvi Vesanen
+Raportointi: Sampsa Näkki
+Jutta Kangas 
 </t>
   </si>
   <si>
@@ -160,10 +162,10 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Eduskuntavaaleista kasvua -  digin ostaminen &amp; operaatiot. avoimuusilmoitus</t>
+      <t xml:space="preserve">Eduskuntavaaleista kasvua -  digin ostaminen &amp; operaatiot. avoimuusilmoitus
+</t>
     </r>
     <r>
       <rPr>
@@ -172,23 +174,11 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
-- vaalituotteistuspaketit myyntikanavasta tekniseen tuotteistukseen vaalipiiri geo-kohdennuksella
+      <t>- vaalituotteistuspaketit myyntikanavasta tekniseen tuotteistukseen vaalipiiri geo-kohdennuksella
 - digi avoimuusilmoitus - DG Tuuli Rikama?
 - aineistoprosessi, digi aineistobannerikoneen linkitys
 - Advendio-Adnuntius integraatio, APIt 
-- luottokorttimaksaminen vs. nykyinen malli laskulla</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-- kampanjaraportti
+- kampanjaraportti, - delivery data &amp; FINA prosessi
 - asiakastuki
 - palevlunhallinta Adnuntius, - consentin ja vendorlistin  päivitys</t>
     </r>
@@ -197,8 +187,8 @@
     <t>Tuuli Rikama</t>
   </si>
   <si>
-    <t>DSE: Bilal Gill, Heidi Falenius, Juho Pöyhönen, Maiju Häkkinen
-DG: Anniina Hautala, Toni Törnqvist, Janne Mikkola, Sini Lähdemäki, Birgitta Kursi, Anu Ollikainen, Rosa Forsell, Jonne Ansamaa, Airi Viljamaa, Mikko Vartiainen
+    <t>DSE: Heidi Falenius, Juho Pöyhönen, Maiju Häkkinen, Hanna Majanmaa, Roope Malho, Anne Salo
+DG: Anniina Hautala, Toni Törnqvist, Janne Mikkonen, Sini Lähdemäki, Birgitta Kursi, Anu Ollikainen, Rosa Forsell, Jonne Ansamaa, Airi Viljamaa, Mikko Vartiainen, Asko Sälli
 MSS: Suvi Vesanen, Jani Moisiola
 TM: Päivi Vaittinen, Niina Grönholm</t>
   </si>
@@ -242,10 +232,10 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Eduskuntavaaleista kasvua -  monimediallinen ostaminen &amp; operaatiot</t>
+      <t xml:space="preserve">Eduskuntavaaleista kasvua -  monimediallinen ostaminen &amp; operaatiot
+</t>
     </r>
     <r>
       <rPr>
@@ -254,8 +244,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
-- Design
+      <t>- Design
 - Ad Manager Print integraatio
 - APIt
 - aineistoilmoitusten monikanavainen generointi ja manageeraus
@@ -266,13 +255,16 @@
     <t>Heidi Falenius</t>
   </si>
   <si>
-    <t>DSE: Antero Karttunen, Vesa Lindqvist
-DG: Anniina Hautala, Toni Törnqvist, Airi Viljamaa, Janne Mikkonen, Sini Lähdemäki
+    <t>DSE: Antero Karttunen, Vesa Lindqvist, Maiju Häkkinen, Roope Malho, Anne Salo
+DG: Anniina Hautala, Toni Törnqvist, Airi Viljamaa, Janne Mikkonen, Sini Lähdemäki, Tuuli Rikama, Jonne Ansamaa, Birgitta Kursi, Anu Ollikainen, Rosa Forsell, 
 MSS: Suvi Vesanen, Jani Moisiola
 TM: Päivi Vaittiinen, Harri Lilja
 N&amp;F: Sanna Wirkkala
-Jaana Tanskanen
-Jero Liimatainen</t>
+Jaana Tanskanen, Asko Sälli, Tuomas Waris
+Jero Liimatainen, Juho Pöyhönen</t>
+  </si>
+  <si>
+    <t>3 h</t>
   </si>
   <si>
     <t>MSS</t>
@@ -553,7 +545,7 @@
     <t>Tuloksellisuus. Yhteiskehittämisen mallin edistäminen S3. Valitut end-to-end yhteiskehittämisen mallin mukaiset pilotit (revops &amp; tuloksellisuuden malli). Miten data tallennetaan, varmistetaan, että toimitaan S3 mallin edistämiseksi fiksusti vaikka sen ympärillä ei teknisempää kehitystä.</t>
   </si>
   <si>
-    <t>Reeta Thurman (Markkinointistrategt), Tiina Virtanen (Solutions Sales), Pilvi Seppälä (Sales dev), Sami Tirkkonen (CX), Hanna Jalonen (Salesdev), Sami Luutiviki (data)</t>
+    <t>Reeta Thurman (Markkinointistrategt), Tiina Virtanen (Solutions Sales), Pilvi Seppälä (Sales dev), Sami Tirkkonen (CX), Hanna Jalonen (Salesdev), Sami Luutikivi (data)</t>
   </si>
   <si>
     <t>0,5</t>
@@ -589,7 +581,7 @@
     <t>Discovery: kasvupalvelun asiakkaiden mainosdatan rikastaminen tulosten parantamiseksi; vaihtoehtojen kartoitus ja pilotointi. Datan parannus melko domainin sisäinen työ, mutta pitää huomioida raportointi ja datayhteys näkökulmasta</t>
   </si>
   <si>
-    <t>John Kronström, TBD</t>
+    <t>John Kronström</t>
   </si>
   <si>
     <r>
@@ -637,15 +629,15 @@
   </si>
   <si>
     <t>MSS Media solutions natiivi: Ria Vaahto, Petra Saikku
-DG: Johannes Hocksell, Jaakko Kuivalainen, Jonne Ansamaa
-N&amp;F: Timo Rinne, Anssi Hämäläinen, Teemu Hauhia, Sanna Wirkkala
+DG: Johannes Hocksell, Jaakko Kuivalainen, (Jonne Ansamaa)
+N&amp;F: Timo Rinne, Anssi Hämäläinen, (Teemu Hauhia, Sanna Wirkkala)
 Yield: Tuukka Antikainen, Aki Salonen</t>
   </si>
   <si>
     <t>1,5h</t>
   </si>
   <si>
-    <t>Ei ti klo 12 jälkeen, jos mahdollista</t>
+    <t>Ei ti klo 12 jälkeen, jos mahdollista, ei tarvita synchhiin suluissa olevia ihmisiä</t>
   </si>
   <si>
     <t>Ratkaisunrakentaja visio --&gt; ei riippuvuussuunnitteluun,  Mikko N. kontaktoi erikseen tarpeiden keskustelua
@@ -807,7 +799,7 @@
     </r>
   </si>
   <si>
-    <t>TM: Anu Linden, Teemu Ihalainen, Laura KAngas
+    <t>TM: Anu Linden, Teemu Ihalainen, Laura Kangas
 DG: Toni Törnqvist, Tuomas Waris, Anniina Hautala, Janne Mikkonen
 MSS: Raatikainen Satu (toimisto kulma)
 DSE: joku CS tiimistä asiakkaan näkökulmaa tuomaan (Maiju tai hänen nimeämä henkilö)?
@@ -931,7 +923,7 @@
     </r>
   </si>
   <si>
-    <t>Ad Manager: Toni Törnqvist, Anniina Hautala; Display team: Emmy Ramsay; Core: Heidi Falenius; CPR: Jonne Ansama; Performance Products: Hannu Häikiö, Johannes Hocksell</t>
+    <t>Ad Manager: Toni Törnqvist, Anniina Hautala. Display team: Emmy Ramsay. Core: Heidi Falenius. CPR: Jonne Ansamaa. Performance Products: Hannu Häikiö, Johannes Hocksell</t>
   </si>
   <si>
     <r>
@@ -959,7 +951,7 @@
     <t>Netta Aavikko</t>
   </si>
   <si>
-    <t>Ad Manager Product, Campaign Performance &amp; Reporting, Performance Products, Product Sales, Marketing, DSE Core Heidi Falenius, Digital Operations
+    <t>DSE: Core Heidi Falenius
 PP: Johannes Hocksell
 CPR: Janne Eränen, Jonne Ansamaa​
 Juho Pöyhönen
@@ -1157,7 +1149,7 @@
     <t>Anu Linden</t>
   </si>
   <si>
-    <t>B2B Core: Hedi Falenius,  Juho Pöyhönen, Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Teemu Ihalainen, Sina Reunala, Petri Lahikainen, Roope Hämäläinen</t>
+    <t>B2B Core: Hedi Falenius,  Juho Pöyhönen, Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Teemu Ihalainen, Sina Reunala, Petri Lahikainen, Roope Hämäläinen, Jukka Siltakorpi</t>
   </si>
   <si>
     <t>2 h</t>
@@ -1206,9 +1198,6 @@
     <t>Campaign performance &amp; Reporting: Jonne Ansamaa, Riia Luhtala, Sari Moilanen, Pilvi Rimmanen
 Core &amp; Sales Reporting: Heidi Falenius, Sampsa Näkki. 
 Total TV &amp; Audio Products​: Anu Linden, Annika Palm, Pia Viinikainen, Joonas Imeläinen, Teemu Ihalainen, Petri Lahikainen, Mikko Eskelinen, Panu Hyryläinen, Sina Reunala, Laura Kangas, Tina Åström</t>
-  </si>
-  <si>
-    <t>3 h</t>
   </si>
 </sst>
 </file>
@@ -2111,26 +2100,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07127F19-9F63-3B48-ABE6-8FC4ADCB9798}">
   <dimension ref="A1:J69"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3" style="37" customWidth="1"/>
-    <col min="2" max="2" width="9" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="2"/>
     <col min="4" max="4" width="87.5" customWidth="1"/>
     <col min="5" max="5" width="18.875" style="34" customWidth="1"/>
-    <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="18.625" customWidth="1"/>
+    <col min="6" max="7" width="58" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="31.5" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="15.5" style="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21">
+    <row r="1" spans="1:10" ht="21.95">
       <c r="D1" s="9" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="32.1">
+    <row r="2" spans="1:10" ht="6.75" customHeight="1"/>
+    <row r="3" spans="1:10" ht="33.950000000000003">
       <c r="B3" s="32" t="s">
         <v>1</v>
       </c>
@@ -2159,7 +2148,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="25.5">
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A4" s="38"/>
       <c r="B4" s="12" t="s">
         <v>10</v>
@@ -2185,7 +2174,7 @@
       </c>
       <c r="J4" s="34"/>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="138.75">
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="117" customHeight="1">
       <c r="A5" s="38"/>
       <c r="B5" s="42" t="s">
         <v>15</v>
@@ -2202,14 +2191,16 @@
       <c r="F5" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="22"/>
+      <c r="G5" s="22">
+        <v>2</v>
+      </c>
       <c r="H5" s="33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="63"/>
       <c r="J5" s="34"/>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="128.1" customHeight="1">
+    <row r="6" spans="1:10" s="1" customFormat="1" ht="140.25" customHeight="1">
       <c r="A6" s="38"/>
       <c r="B6" s="42" t="s">
         <v>19</v>
@@ -2217,7 +2208,7 @@
       <c r="C6" s="14">
         <v>2</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="28" t="s">
         <v>20</v>
       </c>
       <c r="E6" s="22" t="s">
@@ -2235,7 +2226,7 @@
       <c r="I6" s="63"/>
       <c r="J6" s="34"/>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="77.25">
+    <row r="7" spans="1:10" s="1" customFormat="1" ht="119.1">
       <c r="A7" s="38"/>
       <c r="B7" s="42" t="s">
         <v>10</v>
@@ -2261,7 +2252,7 @@
       </c>
       <c r="J7" s="34"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="105">
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="120">
       <c r="A8" s="38"/>
       <c r="B8" s="42" t="s">
         <v>10</v>
@@ -2269,7 +2260,7 @@
       <c r="C8" s="14">
         <v>2</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="28" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="23" t="s">
@@ -2278,32 +2269,34 @@
       <c r="F8" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="22"/>
+      <c r="G8" s="22" t="s">
+        <v>30</v>
+      </c>
       <c r="H8" s="33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="63"/>
       <c r="J8" s="69"/>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="99" customHeight="1">
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="105" customHeight="1">
       <c r="A9" s="38"/>
       <c r="B9" s="26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="39" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H9" s="70" t="b">
         <v>1</v>
@@ -2311,22 +2304,22 @@
       <c r="I9" s="16"/>
       <c r="J9" s="34"/>
     </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="96.95" customHeight="1">
+    <row r="10" spans="1:10" s="1" customFormat="1" ht="119.25" customHeight="1">
       <c r="A10" s="38"/>
       <c r="B10" s="30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="14">
         <v>9</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G10"/>
       <c r="H10" s="33" t="b">
@@ -2335,48 +2328,48 @@
       <c r="I10" s="16"/>
       <c r="J10" s="34"/>
     </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="38.25">
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="120.95" customHeight="1">
       <c r="A11" s="38"/>
       <c r="B11" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" s="15">
         <v>10</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H11" s="33" t="b">
         <v>1</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" s="1" customFormat="1" ht="39">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="1" customFormat="1" ht="117.75" customHeight="1">
       <c r="A12" s="38"/>
       <c r="B12" s="19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" s="23"/>
       <c r="D12" s="24" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G12" s="22"/>
       <c r="H12" s="33" t="b">
@@ -2384,25 +2377,25 @@
       </c>
       <c r="I12" s="16"/>
       <c r="J12" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="1" customFormat="1" ht="45">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="1" customFormat="1" ht="79.5" customHeight="1">
       <c r="A13" s="38"/>
       <c r="B13" s="19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C13" s="23">
         <v>7</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G13" s="22"/>
       <c r="H13" s="33" t="b">
@@ -2411,7 +2404,7 @@
       <c r="I13" s="16"/>
       <c r="J13" s="34"/>
     </row>
-    <row r="14" spans="1:10" s="1" customFormat="1" ht="25.5">
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A14" s="38"/>
       <c r="B14" s="19" t="s">
         <v>10</v>
@@ -2420,24 +2413,24 @@
         <v>11</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E14" s="23"/>
       <c r="F14" s="40" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G14" s="22"/>
       <c r="H14" s="33" t="b">
         <v>0</v>
       </c>
       <c r="I14" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J14" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="25.5">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A15" s="38"/>
       <c r="B15" s="19" t="s">
         <v>10</v>
@@ -2446,24 +2439,24 @@
         <v>10</v>
       </c>
       <c r="D15" s="45" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="22"/>
       <c r="F15" s="41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G15" s="22"/>
       <c r="H15" s="33" t="b">
         <v>0</v>
       </c>
       <c r="I15" s="72" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J15" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="26.1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A16" s="38"/>
       <c r="B16" s="19" t="s">
         <v>10</v>
@@ -2472,13 +2465,13 @@
         <v>10</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G16" s="22"/>
       <c r="H16" s="33" t="b">
@@ -2487,22 +2480,22 @@
       <c r="I16" s="27"/>
       <c r="J16" s="34"/>
     </row>
-    <row r="17" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="17" spans="1:10" s="1" customFormat="1" ht="90.95" customHeight="1">
       <c r="A17" s="38"/>
       <c r="B17" s="26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17" s="15">
         <v>4</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="22"/>
       <c r="H17" s="43" t="b">
@@ -2511,22 +2504,22 @@
       <c r="I17" s="17"/>
       <c r="J17" s="29"/>
     </row>
-    <row r="18" spans="1:10" s="1" customFormat="1" ht="51.95">
+    <row r="18" spans="1:10" s="1" customFormat="1" ht="84" customHeight="1">
       <c r="A18" s="38"/>
       <c r="B18" s="26" t="s">
         <v>15</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G18" s="22"/>
       <c r="H18" s="33" t="b">
@@ -2535,29 +2528,29 @@
       <c r="I18" s="16"/>
       <c r="J18" s="34"/>
     </row>
-    <row r="19" spans="1:10" s="1" customFormat="1" ht="50.25">
+    <row r="19" spans="1:10" s="1" customFormat="1" ht="84" customHeight="1">
       <c r="A19" s="38"/>
       <c r="B19" s="26" t="s">
         <v>15</v>
       </c>
       <c r="C19" s="61" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G19" s="22"/>
       <c r="H19" s="33" t="b">
         <v>1</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J19" s="34"/>
     </row>
@@ -2567,16 +2560,16 @@
         <v>10</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G20" s="22"/>
       <c r="H20" s="33" t="b">
@@ -2584,10 +2577,10 @@
       </c>
       <c r="I20" s="16"/>
       <c r="J20" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" s="1" customFormat="1" ht="38.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A21" s="38"/>
       <c r="B21" s="19" t="s">
         <v>15</v>
@@ -2596,13 +2589,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G21" s="22">
         <v>1</v>
@@ -2611,13 +2604,13 @@
         <v>1</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J21" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" s="1" customFormat="1" ht="26.1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A22" s="38"/>
       <c r="B22" s="19" t="s">
         <v>15</v>
@@ -2626,24 +2619,24 @@
         <v>1</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G22" s="22">
         <v>1</v>
       </c>
       <c r="H22" s="43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" s="16"/>
       <c r="J22" s="34"/>
     </row>
-    <row r="23" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="23" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A23" s="38"/>
       <c r="B23" s="19" t="s">
         <v>15</v>
@@ -2652,16 +2645,16 @@
         <v>1</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H23" s="43" t="b">
         <v>1</v>
@@ -2669,7 +2662,7 @@
       <c r="I23" s="16"/>
       <c r="J23" s="34"/>
     </row>
-    <row r="24" spans="1:10" s="1" customFormat="1" ht="26.1">
+    <row r="24" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A24" s="38"/>
       <c r="B24" s="19" t="s">
         <v>15</v>
@@ -2678,13 +2671,13 @@
         <v>1</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G24" s="22">
         <v>1</v>
@@ -2693,11 +2686,11 @@
         <v>1</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J24" s="34"/>
     </row>
-    <row r="25" spans="1:10" s="1" customFormat="1">
+    <row r="25" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A25" s="38"/>
       <c r="B25" s="19" t="s">
         <v>15</v>
@@ -2706,22 +2699,22 @@
         <v>9</v>
       </c>
       <c r="D25" s="62" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G25" s="22"/>
       <c r="H25" s="43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="34"/>
     </row>
-    <row r="26" spans="1:10" s="1" customFormat="1" ht="25.5">
+    <row r="26" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A26" s="38"/>
       <c r="B26" s="19" t="s">
         <v>15</v>
@@ -2730,24 +2723,24 @@
         <v>9</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G26" s="22"/>
       <c r="H26" s="43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J26" s="34"/>
     </row>
-    <row r="27" spans="1:10" s="1" customFormat="1" ht="25.5">
+    <row r="27" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A27" s="38"/>
       <c r="B27" s="19" t="s">
         <v>15</v>
@@ -2756,24 +2749,24 @@
         <v>9</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G27" s="22"/>
       <c r="H27" s="43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J27" s="34"/>
     </row>
-    <row r="28" spans="1:10" s="1" customFormat="1" ht="15.75">
+    <row r="28" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A28" s="38"/>
       <c r="B28" s="19" t="s">
         <v>15</v>
@@ -2782,26 +2775,26 @@
         <v>9</v>
       </c>
       <c r="D28" s="62" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G28" s="22"/>
       <c r="H28" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I28" s="71" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J28" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" s="1" customFormat="1" ht="26.1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" s="1" customFormat="1" ht="89.25" customHeight="1">
       <c r="A29" s="38"/>
       <c r="B29" s="19" t="s">
         <v>15</v>
@@ -2810,13 +2803,13 @@
         <v>9</v>
       </c>
       <c r="D29" s="62" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G29" s="22"/>
       <c r="H29" s="43" t="b">
@@ -2825,35 +2818,35 @@
       <c r="I29" s="16"/>
       <c r="J29" s="34"/>
     </row>
-    <row r="30" spans="1:10" s="1" customFormat="1" ht="65.25" customHeight="1">
+    <row r="30" spans="1:10" s="1" customFormat="1" ht="73.5" customHeight="1">
       <c r="A30" s="38"/>
       <c r="B30" s="21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30" s="15">
         <v>5</v>
       </c>
       <c r="D30" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F30" s="25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H30" s="43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J30" s="29"/>
     </row>
-    <row r="31" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="31" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A31" s="38"/>
       <c r="B31" s="26" t="s">
         <v>10</v>
@@ -2862,24 +2855,24 @@
         <v>9</v>
       </c>
       <c r="D31" s="44" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E31" s="15"/>
       <c r="F31" s="25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G31" s="22"/>
       <c r="H31" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I31" s="73" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J31" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" s="1" customFormat="1" ht="25.5">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A32" s="38"/>
       <c r="B32" s="26" t="s">
         <v>10</v>
@@ -2888,39 +2881,39 @@
         <v>4</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F32" s="25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H32" s="43" t="b">
         <v>1</v>
       </c>
       <c r="I32" s="36"/>
       <c r="J32" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" s="1" customFormat="1" ht="51.95">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="1" customFormat="1" ht="71.25" customHeight="1">
       <c r="A33" s="38"/>
       <c r="B33" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C33" s="15"/>
       <c r="D33" s="24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F33" s="25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G33" s="22"/>
       <c r="H33" s="43" t="b">
@@ -2929,20 +2922,20 @@
       <c r="I33" s="36"/>
       <c r="J33" s="29"/>
     </row>
-    <row r="34" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="34" spans="1:10" s="1" customFormat="1" ht="63.95" customHeight="1">
       <c r="A34" s="38"/>
       <c r="B34" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C34" s="15"/>
       <c r="D34" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G34" s="22"/>
       <c r="H34" s="43" t="b">
@@ -2951,7 +2944,7 @@
       <c r="I34" s="16"/>
       <c r="J34" s="29"/>
     </row>
-    <row r="35" spans="1:10" s="1" customFormat="1" ht="120">
+    <row r="35" spans="1:10" s="1" customFormat="1" ht="80.25" customHeight="1">
       <c r="A35" s="38"/>
       <c r="B35" s="21" t="s">
         <v>19</v>
@@ -2960,13 +2953,13 @@
         <v>6</v>
       </c>
       <c r="D35" s="28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G35" s="22">
         <v>1</v>
@@ -2975,13 +2968,13 @@
         <v>1</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J35" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" s="1" customFormat="1" ht="120">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" s="1" customFormat="1" ht="63" customHeight="1">
       <c r="A36" s="38"/>
       <c r="B36" s="21" t="s">
         <v>19</v>
@@ -2990,28 +2983,28 @@
         <v>6</v>
       </c>
       <c r="D36" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G36" s="22">
+        <v>1</v>
+      </c>
+      <c r="H36" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="F36" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="G36" s="22">
-        <v>1</v>
-      </c>
-      <c r="H36" s="43" t="b">
-        <v>1</v>
-      </c>
-      <c r="I36" s="16" t="s">
-        <v>117</v>
-      </c>
       <c r="J36" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" s="1" customFormat="1" ht="65.099999999999994">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A37" s="38"/>
       <c r="B37" s="21" t="s">
         <v>19</v>
@@ -3020,13 +3013,13 @@
         <v>7</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G37" s="22">
         <v>1.5</v>
@@ -3037,7 +3030,7 @@
       <c r="I37" s="16"/>
       <c r="J37" s="29"/>
     </row>
-    <row r="38" spans="1:10" s="1" customFormat="1" ht="75.75">
+    <row r="38" spans="1:10" s="1" customFormat="1" ht="63" customHeight="1">
       <c r="A38" s="38"/>
       <c r="B38" s="21" t="s">
         <v>19</v>
@@ -3046,26 +3039,26 @@
         <v>8</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H38" s="43" t="b">
         <v>1</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J38" s="29"/>
     </row>
-    <row r="39" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="39" spans="1:10" s="1" customFormat="1" ht="80.25" customHeight="1">
       <c r="A39" s="38"/>
       <c r="B39" s="21" t="s">
         <v>19</v>
@@ -3074,26 +3067,26 @@
         <v>3</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G39" s="22"/>
       <c r="H39" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J39" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" s="1" customFormat="1" ht="45">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A40" s="38"/>
       <c r="B40" s="21" t="s">
         <v>19</v>
@@ -3102,26 +3095,26 @@
         <v>9</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G40" s="22"/>
       <c r="H40" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J40" s="29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" s="1" customFormat="1" ht="63">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A41" s="38"/>
       <c r="B41" s="21" t="s">
         <v>19</v>
@@ -3130,26 +3123,26 @@
         <v>3</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H41" s="43" t="b">
         <v>1</v>
       </c>
       <c r="I41" s="16"/>
       <c r="J41" s="34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" s="1" customFormat="1" ht="38.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A42" s="38"/>
       <c r="B42" s="21" t="s">
         <v>19</v>
@@ -3158,16 +3151,16 @@
         <v>3</v>
       </c>
       <c r="D42" s="28" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H42" s="43" t="b">
         <v>1</v>
@@ -3175,7 +3168,7 @@
       <c r="I42" s="16"/>
       <c r="J42" s="34"/>
     </row>
-    <row r="43" spans="1:10" s="1" customFormat="1" ht="135">
+    <row r="43" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A43" s="38"/>
       <c r="B43" s="21" t="s">
         <v>19</v>
@@ -3184,13 +3177,13 @@
         <v>3</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G43" s="22"/>
       <c r="H43" s="43" t="b">
@@ -3199,23 +3192,23 @@
       <c r="I43" s="16"/>
       <c r="J43" s="34"/>
     </row>
-    <row r="44" spans="1:10" s="1" customFormat="1" ht="38.25">
+    <row r="44" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A44" s="38"/>
       <c r="B44" s="21" t="s">
         <v>19</v>
       </c>
       <c r="C44" s="15"/>
       <c r="D44" s="49" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H44" s="43" t="b">
         <v>1</v>
@@ -3223,47 +3216,47 @@
       <c r="I44" s="16"/>
       <c r="J44" s="34"/>
     </row>
-    <row r="45" spans="1:10" s="1" customFormat="1">
+    <row r="45" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A45" s="38"/>
       <c r="B45" s="12" t="s">
         <v>19</v>
       </c>
       <c r="C45" s="15"/>
       <c r="D45" s="68" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G45" s="22"/>
       <c r="H45" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I45" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J45" s="34"/>
     </row>
-    <row r="46" spans="1:10" s="1" customFormat="1" ht="15.75">
+    <row r="46" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A46" s="38"/>
       <c r="B46" s="12" t="s">
         <v>19</v>
       </c>
       <c r="C46" s="15"/>
       <c r="D46" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="E46" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="E46" s="15" t="s">
-        <v>145</v>
-      </c>
       <c r="F46" s="16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H46" s="43" t="b">
         <v>1</v>
@@ -3271,71 +3264,71 @@
       <c r="I46" s="16"/>
       <c r="J46" s="34"/>
     </row>
-    <row r="47" spans="1:10" s="1" customFormat="1" ht="51.95">
+    <row r="47" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A47" s="38"/>
       <c r="B47" s="21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C47" s="15"/>
       <c r="D47" s="51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E47" s="52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F47" s="49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G47" s="22"/>
       <c r="H47" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I47" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J47" s="34"/>
     </row>
-    <row r="48" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="48" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A48" s="38"/>
       <c r="B48" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C48" s="15"/>
       <c r="D48" s="51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E48" s="52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F48" s="49" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G48" s="22"/>
       <c r="H48" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I48" s="71" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J48" s="34"/>
     </row>
-    <row r="49" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="49" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A49" s="38"/>
       <c r="B49" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C49" s="15"/>
       <c r="D49" s="51" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E49" s="52" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H49" s="43" t="b">
         <v>1</v>
@@ -3343,23 +3336,23 @@
       <c r="I49" s="60"/>
       <c r="J49" s="34"/>
     </row>
-    <row r="50" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="50" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A50" s="38"/>
-      <c r="B50" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C50" s="15"/>
+      <c r="B50" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C50" s="23"/>
       <c r="D50" s="51" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E50" s="52" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H50" s="43" t="b">
         <v>1</v>
@@ -3367,23 +3360,23 @@
       <c r="I50" s="60"/>
       <c r="J50" s="34"/>
     </row>
-    <row r="51" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="51" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A51" s="38"/>
-      <c r="B51" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C51" s="15"/>
+      <c r="B51" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C51" s="23"/>
       <c r="D51" s="51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E51" s="52" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H51" s="43" t="b">
         <v>1</v>
@@ -3391,23 +3384,23 @@
       <c r="I51" s="60"/>
       <c r="J51" s="34"/>
     </row>
-    <row r="52" spans="1:10" s="1" customFormat="1" ht="30">
+    <row r="52" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A52" s="38"/>
-      <c r="B52" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C52" s="15"/>
+      <c r="B52" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C52" s="23"/>
       <c r="D52" s="51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E52" s="52" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H52" s="43" t="b">
         <v>1</v>
@@ -3415,23 +3408,23 @@
       <c r="I52" s="60"/>
       <c r="J52" s="34"/>
     </row>
-    <row r="53" spans="1:10" s="1" customFormat="1" ht="39">
+    <row r="53" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A53" s="38"/>
       <c r="B53" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C53" s="15"/>
       <c r="D53" s="51" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E53" s="52" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F53" s="49" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H53" s="43" t="b">
         <v>1</v>
@@ -3439,47 +3432,47 @@
       <c r="I53" s="60"/>
       <c r="J53" s="34"/>
     </row>
-    <row r="54" spans="1:10" s="1" customFormat="1" ht="104.1">
+    <row r="54" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A54" s="38"/>
       <c r="B54" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C54" s="15"/>
       <c r="D54" s="51" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E54" s="52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F54" s="49" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G54" s="22"/>
       <c r="H54" s="43" t="b">
         <v>0</v>
       </c>
       <c r="I54" s="75" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J54" s="34"/>
     </row>
-    <row r="55" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="55" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A55" s="38"/>
       <c r="B55" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C55" s="15"/>
       <c r="D55" s="51" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E55" s="52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F55" s="49" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H55" s="43" t="b">
         <v>1</v>
@@ -3487,23 +3480,23 @@
       <c r="I55" s="60"/>
       <c r="J55" s="34"/>
     </row>
-    <row r="56" spans="1:10" s="1" customFormat="1" ht="30">
+    <row r="56" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A56" s="38"/>
-      <c r="B56" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C56" s="15"/>
+      <c r="B56" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C56" s="23"/>
       <c r="D56" s="51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E56" s="52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F56" s="49" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H56" s="43" t="b">
         <v>1</v>
@@ -3511,19 +3504,19 @@
       <c r="I56" s="60"/>
       <c r="J56" s="34"/>
     </row>
-    <row r="57" spans="1:10" s="1" customFormat="1">
+    <row r="57" spans="1:10" s="1" customFormat="1" ht="78" customHeight="1">
       <c r="A57" s="38"/>
       <c r="B57" s="12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C57" s="15">
         <v>10</v>
       </c>
       <c r="D57" s="51" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E57" s="52" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F57" s="53"/>
       <c r="G57" s="22"/>
@@ -3531,27 +3524,27 @@
         <v>0</v>
       </c>
       <c r="I57" s="74" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J57" s="34"/>
     </row>
-    <row r="58" spans="1:10" s="1" customFormat="1" ht="78">
+    <row r="58" spans="1:10" s="1" customFormat="1" ht="104.25" customHeight="1">
       <c r="A58" s="38"/>
       <c r="B58" s="47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C58" s="15"/>
       <c r="D58" s="51" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E58" s="52" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F58" s="48" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="H58" s="43" t="b">
         <v>1</v>
@@ -3559,7 +3552,7 @@
       <c r="I58" s="60"/>
       <c r="J58" s="34"/>
     </row>
-    <row r="59" spans="1:10" s="1" customFormat="1">
+    <row r="59" spans="1:10" s="1" customFormat="1" ht="15.95">
       <c r="A59" s="38"/>
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
@@ -3571,7 +3564,7 @@
       <c r="I59" s="11"/>
       <c r="J59" s="34"/>
     </row>
-    <row r="60" spans="1:10" s="1" customFormat="1">
+    <row r="60" spans="1:10" s="1" customFormat="1" ht="15.95">
       <c r="A60" s="38"/>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
@@ -3582,7 +3575,7 @@
       <c r="I60" s="8"/>
       <c r="J60" s="34"/>
     </row>
-    <row r="61" spans="1:10" s="1" customFormat="1" ht="18.600000000000001">
+    <row r="61" spans="1:10" s="1" customFormat="1" ht="18.95">
       <c r="A61" s="38"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -3594,7 +3587,7 @@
       <c r="I61" s="4"/>
       <c r="J61" s="34"/>
     </row>
-    <row r="62" spans="1:10" ht="18.600000000000001">
+    <row r="62" spans="1:10" ht="18.95">
       <c r="B62" s="5"/>
       <c r="C62" s="5"/>
       <c r="D62" s="6"/>
@@ -3604,7 +3597,7 @@
       <c r="H62" s="6"/>
       <c r="I62" s="6"/>
     </row>
-    <row r="63" spans="1:10" ht="18.600000000000001">
+    <row r="63" spans="1:10" ht="18.95">
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
       <c r="D63" s="6"/>
@@ -3614,7 +3607,7 @@
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
     </row>
-    <row r="64" spans="1:10" ht="18.600000000000001">
+    <row r="64" spans="1:10" ht="18.95">
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
       <c r="D64" s="6"/>
@@ -3624,7 +3617,7 @@
       <c r="H64" s="6"/>
       <c r="I64" s="6"/>
     </row>
-    <row r="65" spans="2:9" ht="18.600000000000001">
+    <row r="65" spans="2:9" ht="18.95">
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
       <c r="D65" s="6"/>
@@ -3634,7 +3627,7 @@
       <c r="H65" s="6"/>
       <c r="I65" s="6"/>
     </row>
-    <row r="66" spans="2:9" ht="18.600000000000001">
+    <row r="66" spans="2:9" ht="18.95">
       <c r="B66" s="5"/>
       <c r="C66" s="5"/>
       <c r="D66" s="6"/>
@@ -3644,7 +3637,7 @@
       <c r="H66" s="6"/>
       <c r="I66" s="6"/>
     </row>
-    <row r="67" spans="2:9" ht="18.600000000000001">
+    <row r="67" spans="2:9" ht="18.95">
       <c r="B67" s="5"/>
       <c r="C67" s="5"/>
       <c r="D67" s="6"/>
@@ -3654,7 +3647,7 @@
       <c r="H67" s="6"/>
       <c r="I67" s="6"/>
     </row>
-    <row r="68" spans="2:9" ht="18.600000000000001">
+    <row r="68" spans="2:9" ht="18.95">
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
       <c r="D68" s="6"/>
@@ -3664,7 +3657,7 @@
       <c r="H68" s="6"/>
       <c r="I68" s="6"/>
     </row>
-    <row r="69" spans="2:9" ht="18.600000000000001">
+    <row r="69" spans="2:9" ht="18.95">
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
       <c r="D69" s="6"/>
@@ -3696,15 +3689,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006958AF0A0D18DD46AA2F05B0B7FB2051" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7cc4835c91b31b9b519dddda0e0127ea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8743faf2-653b-47e5-938e-a3c18a0572b2" xmlns:ns3="65bb3d2a-ea9e-471d-8113-08ea35fd4d0a" xmlns:ns4="f0974581-4bbf-443e-902f-14073e9fb4f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b07298893fe1b0d1a251a8914f437576" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="8743faf2-653b-47e5-938e-a3c18a0572b2"/>
@@ -3990,14 +3974,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58C97B2E-9E09-49C0-88E7-D25203A87982}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE028EC4-4BAF-4D78-8C7F-C3E8970CA932}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{113860E7-0903-4CD1-86F2-CB3C963E0E6D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{113860E7-0903-4CD1-86F2-CB3C963E0E6D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE028EC4-4BAF-4D78-8C7F-C3E8970CA932}"/>
 </file>
</xml_diff>